<commit_message>
feat: add INI camera action effects
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -12,8 +12,8 @@
     <sheet name="简体中文" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'English'!$A$1:$I$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'简体中文'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'English'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'简体中文'!$A$1:$I$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -659,8 +659,243 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterAt</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>worldX,worldY</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Centers the local owning player's camera at an absolute world coordinate.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterAt: 400,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>cameraCenterBy</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>deltaX,deltaY</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Moves the local owning player's camera center by a world-space offset.</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>cameraCenterBy: 80,-40</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterOn</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>self|target|actionTarget[,offsetX,offsetY]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Centers the camera on the acting unit, unit target, or action target point with an optional offset.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterOn: actionTarget,0,-60</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>cameraTargetZoom</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>positive float</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Sets the local owning player's native smoothed camera zoom target.</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>cameraTargetZoom: 1.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>cameraStopMovement</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Clears native camera scroll momentum when the action executes.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>cameraStopMovement: true</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -671,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -779,8 +1014,243 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterAt</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>worldX,worldY</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>将本机单位所属玩家的视角中心移动到绝对世界坐标。</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterAt: 400,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>cameraCenterBy</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>deltaX,deltaY</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>按照世界坐标偏移量移动本机单位所属玩家的视角中心。</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>cameraCenterBy: 80,-40</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterOn</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>self|target|actionTarget[,offsetX,offsetY]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>将视角居中到动作单位、目标单位或动作目标点，并可附加坐标偏移。</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>cameraCenterOn: actionTarget,0,-60</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>cameraTargetZoom</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>positive float</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>设置本机单位所属玩家的原版平滑视角缩放目标。</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>cameraTargetZoom: 1.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>cameraStopMovement</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>[action_*] / [hiddenAction_*]</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>new_action_effect</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>client_only</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>在动作执行时清除原版摄像机的滚动惯性。</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>cameraStopMovement: true</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enrich INI damage event context
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -10,10 +10,14 @@
     <sheet name="About 关于" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="English" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="简体中文" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Event Data English" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Event Data 中文" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'English'!$A$1:$I$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'简体中文'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Event Data English'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Event Data 中文'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -477,14 +481,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated from the tracked fields.csv catalog. Do not edit this workbook as the source.</t>
+          <t>Generated from the tracked fields.csv and event-data.csv catalogs. Do not edit this workbook as the source.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>本表由仓库内的 fields.csv 自动生成，请勿把此工作簿作为源文件直接修改。</t>
+          <t>本表由仓库内的 fields.csv 和 event-data.csv 自动生成，请勿把此工作簿作为源文件直接修改。</t>
         </is>
       </c>
     </row>
@@ -1253,4 +1257,866 @@
   <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Version Added</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>eventData Name</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Value Type</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Multiplayer Impact</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Description and usage</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Damage delivered to the native damage routine after attachment forwarding immunity and custom-unit armour.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="damage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>rawDamage</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Damage passed into this custom unit before attachment forwarding immunity and custom-unit armour.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="rawDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>hpDamage</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Actual non-negative HP reduction produced by this damage application.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="hpDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>shieldDamage</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Actual non-negative shield reduction produced by this damage application.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="shieldDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>remainingDamage</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Native return value containing damage left unapplied after shield and hull processing.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="remainingDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>hpBefore</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>HP immediately before the native damage routine.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="hpBefore", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>hpAfter</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>HP immediately after the native damage routine.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="hpAfter", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>shieldBefore</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Shield immediately before the native damage routine.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="shieldBefore", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>shieldAfter</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Shield immediately after the native damage routine.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="shieldAfter", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>wasLethal</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>True when a unit with positive HP reached zero or lower during this damage application.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="wasLethal", type="boolean")</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>加入版本</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>事件</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>eventData 名称</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>值类型</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>联机影响</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>说明与用法</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>传入原版伤害流程的数值；已经过附件伤害转移、伤害免疫和自定义单位护甲处理。</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="damage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>rawDamage</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>最初传入该自定义单位的伤害值；尚未经过附件伤害转移、伤害免疫和自定义单位护甲处理。</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="rawDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>hpDamage</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>本次伤害实际造成的非负生命值减少量。</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="hpDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>shieldDamage</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>本次伤害实际造成的非负护盾值减少量。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="shieldDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>remainingDamage</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>护盾和生命处理结束后未被应用的剩余伤害，即原版伤害方法的返回值。</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="remainingDamage", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>hpBefore</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>进入原版伤害流程前的生命值。</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="hpBefore", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>hpAfter</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>完成原版伤害流程后的生命值。</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="hpAfter", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>shieldBefore</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>进入原版伤害流程前的护盾值。</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="shieldBefore", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>shieldAfter</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>完成原版伤害流程后的护盾值。</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>eventData(name="shieldAfter", type="number")</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>tookDamage</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>wasLethal</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>gameplay_synced</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>若单位在本次伤害前生命值大于零并在之后降到零或更低，则为 true。</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>eventData(name="wasLethal", type="boolean")</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: use shape links in INI reference
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -11,7 +11,18 @@
     <sheet name="English" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="简体中文" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="rf_en_shortcuts">'English'!$A$3</definedName>
+    <definedName name="rf_en_title">'English'!$A$1</definedName>
+    <definedName name="rf_en_core">'English'!$A$6</definedName>
+    <definedName name="rf_en_action">'English'!$A$10</definedName>
+    <definedName name="rf_en_took_damage_event_data">'English'!$A$18</definedName>
+    <definedName name="rf_zh_shortcuts">'简体中文'!$A$3</definedName>
+    <definedName name="rf_zh_title">'简体中文'!$A$1</definedName>
+    <definedName name="rf_zh_core">'简体中文'!$A$6</definedName>
+    <definedName name="rf_zh_action">'简体中文'!$A$10</definedName>
+    <definedName name="rf_zh_took_damage_event_data">'简体中文'!$A$18</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,13 +58,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
@@ -74,13 +78,6 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -221,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -232,81 +229,63 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -383,6 +362,595 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="open_rf_en_title">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1047750" y="2971800"/>
+          <a:ext cx="13220700" cy="400050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="open_rf_zh_title">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1047750" y="3371850"/>
+          <a:ext cx="13220700" cy="400050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="shortcut_en_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1219200"/>
+          <a:ext cx="2962275" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="shortcut_en_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="1219200"/>
+          <a:ext cx="8677275" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="shortcut_en_took_damage_event_data">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11639550" y="1219200"/>
+          <a:ext cx="4210050" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="back_en_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14268450" y="1752600"/>
+          <a:ext cx="1581150" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="back_en_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14268450" y="3190875"/>
+          <a:ext cx="1581150" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="back_en_took_damage_event_data">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14268450" y="6267450"/>
+          <a:ext cx="1581150" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="shortcut_zh_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1219200"/>
+          <a:ext cx="2962275" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="shortcut_zh_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2962275" y="1219200"/>
+          <a:ext cx="8677275" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="shortcut_zh_took_damage_event_data">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11639550" y="1219200"/>
+          <a:ext cx="4210050" cy="342900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="back_zh_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14268450" y="1752600"/>
+          <a:ext cx="1581150" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="back_zh_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14268450" y="3143250"/>
+          <a:ext cx="1581150" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="back_zh_took_damage_event_data">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14268450" y="5981700"/>
+          <a:ext cx="1581150" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p/>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -791,23 +1359,23 @@
           <t>Open English reference / 打开英文代码表</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
     </row>
     <row r="11" ht="31" customHeight="1">
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>打开简体中文代码表 / Open Chinese reference</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -821,11 +1389,8 @@
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="B11:G11"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B10" location="'English'!A1" display="Open English reference / 打开英文代码表"/>
-    <hyperlink ref="B11" location="'简体中文'!A1" display="打开简体中文代码表 / Open Chinese reference"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdRFNavigation"/>
 </worksheet>
 </file>
 
@@ -849,952 +1414,952 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>INI Essentials Unit Modding Reference</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="8" t="n"/>
-      <c r="G1" s="8" t="n"/>
-      <c r="H1" s="8" t="n"/>
+      <c r="B1" s="6" t="n"/>
+      <c r="C1" s="6" t="n"/>
+      <c r="D1" s="6" t="n"/>
+      <c r="E1" s="6" t="n"/>
+      <c r="F1" s="6" t="n"/>
+      <c r="G1" s="6" t="n"/>
+      <c r="H1" s="6" t="n"/>
     </row>
     <row r="2" ht="29" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Generated from tracked CSV catalogs. Section colors follow the original Rusted Warfare reference.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Section shortcuts — click to jump</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>tookDamage — eventData(...)</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Core unit functions and opt-in static unit fields</t>
         </is>
       </c>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="7" ht="31" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Version Added</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G7" s="20" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>allowNegativeHp</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Allows overkill damage to leave this custom unit with HP below zero instead of clamping it to zero.</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>allowNegativeHp: true</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>new_key</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="H8" s="21" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>Action effects that run through the native custom-action chain</t>
         </is>
       </c>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="26" t="inlineStr">
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="11" ht="31" customHeight="1">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Version Added</t>
         </is>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D11" s="27" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G11" s="27" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H11" s="27" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>cameraCenterAt</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>worldX,worldY</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Centers the local owning player's camera at an absolute world coordinate.</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>cameraCenterAt: 400,600</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>cameraCenterBy</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>deltaX,deltaY</t>
         </is>
       </c>
-      <c r="D13" s="30" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>Moves the local owning player's camera center by a world-space offset.</t>
         </is>
       </c>
-      <c r="E13" s="30" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>cameraCenterBy: 80,-40</t>
         </is>
       </c>
-      <c r="F13" s="28" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G13" s="28" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H13" s="28" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>cameraCenterOn</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>self|target|actionTarget[,offsetX,offsetY]</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Centers the camera on the acting unit, unit target, or action target point with an optional offset.</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>cameraCenterOn: actionTarget,0,-60</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>cameraTargetZoom</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>positive float</t>
         </is>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>Sets the local owning player's native smoothed camera zoom target.</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>cameraTargetZoom: 1.25</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr">
+      <c r="G15" s="22" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H15" s="28" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>cameraStopMovement</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Clears native camera scroll momentum when the action executes.</t>
         </is>
       </c>
-      <c r="E16" s="23" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>cameraStopMovement: true</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="25" t="inlineStr">
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>tookDamage — eventData(...)</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>Extra context values for the native tookDamage action event</t>
         </is>
       </c>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="26" t="inlineStr">
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="19" ht="31" customHeight="1">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Version Added</t>
         </is>
       </c>
-      <c r="B19" s="27" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D19" s="27" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E19" s="27" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F19" s="27" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G19" s="27" t="inlineStr">
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H19" s="27" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>Damage delivered to the native damage routine after attachment forwarding immunity and custom-unit armour.</t>
         </is>
       </c>
-      <c r="E20" s="23" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>eventData(name="damage", type="number")</t>
         </is>
       </c>
-      <c r="F20" s="21" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>rawDamage</t>
         </is>
       </c>
-      <c r="C21" s="28" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>Damage passed into this custom unit before attachment forwarding immunity and custom-unit armour.</t>
         </is>
       </c>
-      <c r="E21" s="30" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>eventData(name="rawDamage", type="number")</t>
         </is>
       </c>
-      <c r="F21" s="28" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G21" s="28" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H21" s="28" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>hpDamage</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Actual non-negative HP reduction produced by this damage application.</t>
         </is>
       </c>
-      <c r="E22" s="23" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>eventData(name="hpDamage", type="number")</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G22" s="21" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>shieldDamage</t>
         </is>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D23" s="30" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>Actual non-negative shield reduction produced by this damage application.</t>
         </is>
       </c>
-      <c r="E23" s="30" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>eventData(name="shieldDamage", type="number")</t>
         </is>
       </c>
-      <c r="F23" s="28" t="inlineStr">
+      <c r="F23" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G23" s="28" t="inlineStr">
+      <c r="G23" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H23" s="28" t="inlineStr">
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>remainingDamage</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>Native return value containing damage left unapplied after shield and hull processing.</t>
         </is>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>eventData(name="remainingDamage", type="number")</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G24" s="21" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>hpBefore</t>
         </is>
       </c>
-      <c r="C25" s="28" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="24" t="inlineStr">
         <is>
           <t>HP immediately before the native damage routine.</t>
         </is>
       </c>
-      <c r="E25" s="30" t="inlineStr">
+      <c r="E25" s="24" t="inlineStr">
         <is>
           <t>eventData(name="hpBefore", type="number")</t>
         </is>
       </c>
-      <c r="F25" s="28" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G25" s="28" t="inlineStr">
+      <c r="G25" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H25" s="28" t="inlineStr">
+      <c r="H25" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>hpAfter</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>HP immediately after the native damage routine.</t>
         </is>
       </c>
-      <c r="E26" s="23" t="inlineStr">
+      <c r="E26" s="18" t="inlineStr">
         <is>
           <t>eventData(name="hpAfter", type="number")</t>
         </is>
       </c>
-      <c r="F26" s="21" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G26" s="21" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H26" s="21" t="inlineStr">
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>shieldBefore</t>
         </is>
       </c>
-      <c r="C27" s="28" t="inlineStr">
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D27" s="30" t="inlineStr">
+      <c r="D27" s="24" t="inlineStr">
         <is>
           <t>Shield immediately before the native damage routine.</t>
         </is>
       </c>
-      <c r="E27" s="30" t="inlineStr">
+      <c r="E27" s="24" t="inlineStr">
         <is>
           <t>eventData(name="shieldBefore", type="number")</t>
         </is>
       </c>
-      <c r="F27" s="28" t="inlineStr">
+      <c r="F27" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G27" s="28" t="inlineStr">
+      <c r="G27" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H27" s="28" t="inlineStr">
+      <c r="H27" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>shieldAfter</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D28" s="23" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>Shield immediately after the native damage routine.</t>
         </is>
       </c>
-      <c r="E28" s="23" t="inlineStr">
+      <c r="E28" s="18" t="inlineStr">
         <is>
           <t>eventData(name="shieldAfter", type="number")</t>
         </is>
       </c>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G28" s="21" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H28" s="21" t="inlineStr">
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>wasLethal</t>
         </is>
       </c>
-      <c r="C29" s="28" t="inlineStr">
+      <c r="C29" s="22" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="D29" s="30" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>True when a unit with positive HP reached zero or lower during this damage application.</t>
         </is>
       </c>
-      <c r="E29" s="30" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>eventData(name="wasLethal", type="boolean")</t>
         </is>
       </c>
-      <c r="F29" s="28" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G29" s="28" t="inlineStr">
+      <c r="G29" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H29" s="28" t="inlineStr">
+      <c r="H29" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
@@ -1812,17 +2377,10 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E6:G6"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A4" location="'English'!A6" display="[core]"/>
-    <hyperlink ref="C4" location="'English'!A10" display="[action_NAME] / [hiddenAction_NAME]"/>
-    <hyperlink ref="F4" location="'English'!A18" display="tookDamage — eventData(...)"/>
-    <hyperlink ref="H6" location="'English'!A3" display="↑ Shortcuts"/>
-    <hyperlink ref="H10" location="'English'!A3" display="↑ Shortcuts"/>
-    <hyperlink ref="H18" location="'English'!A3" display="↑ Shortcuts"/>
-  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdRFNavigation"/>
 </worksheet>
 </file>
 
@@ -1846,952 +2404,952 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>INI Essentials 单位模组代码表</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="8" t="n"/>
-      <c r="G1" s="8" t="n"/>
-      <c r="H1" s="8" t="n"/>
+      <c r="B1" s="6" t="n"/>
+      <c r="C1" s="6" t="n"/>
+      <c r="D1" s="6" t="n"/>
+      <c r="E1" s="6" t="n"/>
+      <c r="F1" s="6" t="n"/>
+      <c r="G1" s="6" t="n"/>
+      <c r="H1" s="6" t="n"/>
     </row>
     <row r="2" ht="29" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>由仓库内 CSV 代码表生成；各节颜色沿用原版 Rusted Warfare 代码表。</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>节快捷导航——点击即可跳转</t>
         </is>
       </c>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>tookDamage — eventData(...) 事件数据</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>版本</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>单位核心功能与可选的静态单位字段</t>
         </is>
       </c>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="7" ht="31" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>加入版本</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G7" s="20" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>allowNegativeHp</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>允许过量伤害使此自定义单位的生命值降到零以下，而不是夹到零。</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>allowNegativeHp: true</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>new_key</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="H8" s="21" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>版本</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>通过原版自定义动作链执行的动作效果</t>
         </is>
       </c>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="26" t="inlineStr">
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="11" ht="31" customHeight="1">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>加入版本</t>
         </is>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D11" s="27" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G11" s="27" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H11" s="27" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>cameraCenterAt</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>worldX,worldY</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>将本机单位所属玩家的视角中心移动到绝对世界坐标。</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>cameraCenterAt: 400,600</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>cameraCenterBy</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>deltaX,deltaY</t>
         </is>
       </c>
-      <c r="D13" s="30" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>按照世界坐标偏移量移动本机单位所属玩家的视角中心。</t>
         </is>
       </c>
-      <c r="E13" s="30" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>cameraCenterBy: 80,-40</t>
         </is>
       </c>
-      <c r="F13" s="28" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G13" s="28" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H13" s="28" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>cameraCenterOn</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>self|target|actionTarget[,offsetX,offsetY]</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>将视角居中到动作单位、目标单位或动作目标点，并可附加坐标偏移。</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>cameraCenterOn: actionTarget,0,-60</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>cameraTargetZoom</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>positive float</t>
         </is>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>设置本机单位所属玩家的原版平滑视角缩放目标。</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>cameraTargetZoom: 1.25</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr">
+      <c r="G15" s="22" t="inlineStr">
         <is>
           <t>omitted</t>
         </is>
       </c>
-      <c r="H15" s="28" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>cameraStopMovement</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>在动作执行时清除原版摄像机的滚动惯性。</t>
         </is>
       </c>
-      <c r="E16" s="23" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>cameraStopMovement: true</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>new_action_effect</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>client_only</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>版本</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="25" t="inlineStr">
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>tookDamage — eventData(...) 事件数据</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>为原版 tookDamage 动作事件补充的上下文值</t>
         </is>
       </c>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="26" t="inlineStr">
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="19" ht="31" customHeight="1">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>加入版本</t>
         </is>
       </c>
-      <c r="B19" s="27" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D19" s="27" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E19" s="27" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F19" s="27" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G19" s="27" t="inlineStr">
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H19" s="27" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>damage</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>传入原版伤害流程的数值；已经过附件伤害转移、伤害免疫和自定义单位护甲处理。</t>
         </is>
       </c>
-      <c r="E20" s="23" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>eventData(name="damage", type="number")</t>
         </is>
       </c>
-      <c r="F20" s="21" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>rawDamage</t>
         </is>
       </c>
-      <c r="C21" s="28" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>最初传入该自定义单位的伤害值；尚未经过附件伤害转移、伤害免疫和自定义单位护甲处理。</t>
         </is>
       </c>
-      <c r="E21" s="30" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>eventData(name="rawDamage", type="number")</t>
         </is>
       </c>
-      <c r="F21" s="28" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G21" s="28" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H21" s="28" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>hpDamage</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>本次伤害实际造成的非负生命值减少量。</t>
         </is>
       </c>
-      <c r="E22" s="23" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>eventData(name="hpDamage", type="number")</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G22" s="21" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>shieldDamage</t>
         </is>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D23" s="30" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>本次伤害实际造成的非负护盾值减少量。</t>
         </is>
       </c>
-      <c r="E23" s="30" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>eventData(name="shieldDamage", type="number")</t>
         </is>
       </c>
-      <c r="F23" s="28" t="inlineStr">
+      <c r="F23" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G23" s="28" t="inlineStr">
+      <c r="G23" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H23" s="28" t="inlineStr">
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>remainingDamage</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>护盾和生命处理结束后未被应用的剩余伤害，即原版伤害方法的返回值。</t>
         </is>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>eventData(name="remainingDamage", type="number")</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G24" s="21" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>hpBefore</t>
         </is>
       </c>
-      <c r="C25" s="28" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="24" t="inlineStr">
         <is>
           <t>进入原版伤害流程前的生命值。</t>
         </is>
       </c>
-      <c r="E25" s="30" t="inlineStr">
+      <c r="E25" s="24" t="inlineStr">
         <is>
           <t>eventData(name="hpBefore", type="number")</t>
         </is>
       </c>
-      <c r="F25" s="28" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G25" s="28" t="inlineStr">
+      <c r="G25" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H25" s="28" t="inlineStr">
+      <c r="H25" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>hpAfter</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>完成原版伤害流程后的生命值。</t>
         </is>
       </c>
-      <c r="E26" s="23" t="inlineStr">
+      <c r="E26" s="18" t="inlineStr">
         <is>
           <t>eventData(name="hpAfter", type="number")</t>
         </is>
       </c>
-      <c r="F26" s="21" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G26" s="21" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H26" s="21" t="inlineStr">
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>shieldBefore</t>
         </is>
       </c>
-      <c r="C27" s="28" t="inlineStr">
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D27" s="30" t="inlineStr">
+      <c r="D27" s="24" t="inlineStr">
         <is>
           <t>进入原版伤害流程前的护盾值。</t>
         </is>
       </c>
-      <c r="E27" s="30" t="inlineStr">
+      <c r="E27" s="24" t="inlineStr">
         <is>
           <t>eventData(name="shieldBefore", type="number")</t>
         </is>
       </c>
-      <c r="F27" s="28" t="inlineStr">
+      <c r="F27" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G27" s="28" t="inlineStr">
+      <c r="G27" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H27" s="28" t="inlineStr">
+      <c r="H27" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>shieldAfter</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D28" s="23" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>完成原版伤害流程后的护盾值。</t>
         </is>
       </c>
-      <c r="E28" s="23" t="inlineStr">
+      <c r="E28" s="18" t="inlineStr">
         <is>
           <t>eventData(name="shieldAfter", type="number")</t>
         </is>
       </c>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G28" s="21" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H28" s="21" t="inlineStr">
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>wasLethal</t>
         </is>
       </c>
-      <c r="C29" s="28" t="inlineStr">
+      <c r="C29" s="22" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="D29" s="30" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>若单位在本次伤害前生命值大于零并在之后降到零或更低，则为 true。</t>
         </is>
       </c>
-      <c r="E29" s="30" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>eventData(name="wasLethal", type="boolean")</t>
         </is>
       </c>
-      <c r="F29" s="28" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>native_event_data</t>
         </is>
       </c>
-      <c r="G29" s="28" t="inlineStr">
+      <c r="G29" s="22" t="inlineStr">
         <is>
           <t>available during event</t>
         </is>
       </c>
-      <c r="H29" s="28" t="inlineStr">
+      <c r="H29" s="22" t="inlineStr">
         <is>
           <t>gameplay_synced</t>
         </is>
@@ -2809,16 +3367,9 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E6:G6"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A4" location="'简体中文'!A6" display="[core]"/>
-    <hyperlink ref="C4" location="'简体中文'!A10" display="[action_NAME] / [hiddenAction_NAME]"/>
-    <hyperlink ref="F4" location="'简体中文'!A18" display="tookDamage — eventData(...) 事件数据"/>
-    <hyperlink ref="H6" location="'简体中文'!A3" display="↑ 返回节导航"/>
-    <hyperlink ref="H10" location="'简体中文'!A3" display="↑ 返回节导航"/>
-    <hyperlink ref="H18" location="'简体中文'!A3" display="↑ 返回节导航"/>
-  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdRFNavigation"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make INI extension values runtime expressions
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -2994,7 +2994,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="3857625"/>
+          <a:off x="14268450" y="3905250"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3035,7 +3035,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="7419975"/>
+          <a:off x="14268450" y="7562850"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3076,7 +3076,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="13877925"/>
+          <a:off x="14268450" y="14020800"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3117,7 +3117,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="17078325"/>
+          <a:off x="14268450" y="17221200"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3158,7 +3158,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="27689175"/>
+          <a:off x="0" y="27832050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3215,7 +3215,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="27689175"/>
+          <a:off x="3962400" y="27832050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3272,7 +3272,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="27689175"/>
+          <a:off x="7924800" y="27832050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3329,7 +3329,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="27689175"/>
+          <a:off x="11887200" y="27832050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3386,7 +3386,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="28032075"/>
+          <a:off x="0" y="28174950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3443,7 +3443,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="28032075"/>
+          <a:off x="3962400" y="28174950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3500,7 +3500,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="28032075"/>
+          <a:off x="7924800" y="28174950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3557,7 +3557,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="28032075"/>
+          <a:off x="11887200" y="28174950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3614,7 +3614,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="28374975"/>
+          <a:off x="0" y="28517850"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3671,7 +3671,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="28374975"/>
+          <a:off x="3962400" y="28517850"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3728,7 +3728,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="28374975"/>
+          <a:off x="7924800" y="28517850"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3785,7 +3785,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="28374975"/>
+          <a:off x="11887200" y="28517850"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3842,7 +3842,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="28717875"/>
+          <a:off x="0" y="28860750"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3899,7 +3899,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="28717875"/>
+          <a:off x="3962400" y="28860750"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3956,7 +3956,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="28717875"/>
+          <a:off x="7924800" y="28860750"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4013,7 +4013,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="29251275"/>
+          <a:off x="14268450" y="29394150"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4054,7 +4054,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="33899475"/>
+          <a:off x="14268450" y="34042350"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4095,7 +4095,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="38690550"/>
+          <a:off x="14268450" y="38833425"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4136,7 +4136,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="43481625"/>
+          <a:off x="14268450" y="43624500"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4177,7 +4177,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="47186850"/>
+          <a:off x="14268450" y="47329725"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4218,7 +4218,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="49663350"/>
+          <a:off x="14268450" y="49806225"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4259,7 +4259,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="53587650"/>
+          <a:off x="14268450" y="53730525"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4300,7 +4300,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="56111775"/>
+          <a:off x="14268450" y="56254650"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4341,7 +4341,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="60083700"/>
+          <a:off x="14268450" y="60226575"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4382,7 +4382,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="63646050"/>
+          <a:off x="14268450" y="63788925"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4423,7 +4423,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="66484500"/>
+          <a:off x="14268450" y="66627375"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4464,7 +4464,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="70046850"/>
+          <a:off x="14268450" y="70189725"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4505,7 +4505,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="73609200"/>
+          <a:off x="14268450" y="73752075"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4546,7 +4546,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="77171550"/>
+          <a:off x="14268450" y="77314425"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4587,7 +4587,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="80733900"/>
+          <a:off x="14268450" y="80876775"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5244,17 +5244,17 @@
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>runtime LogicBoolean</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>Allows overkill damage to leave this custom unit with HP below zero instead of clamping it to zero.</t>
+          <t>Allows overkill damage to leave this custom unit with HP below zero whenever the runtime condition is true.</t>
         </is>
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>allowNegativeHp: true</t>
+          <t>allowNegativeHp: memory.berserk or self.resource.rage &gt; 0</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
@@ -5358,17 +5358,17 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>worldX,worldY</t>
+          <t>runtimeNumberX,runtimeNumberY</t>
         </is>
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Centers the local owning player's camera at an absolute world coordinate.</t>
+          <t>Centers the local owning player's camera at runtime-evaluated absolute world coordinates.</t>
         </is>
       </c>
       <c r="E14" s="22" t="inlineStr">
         <is>
-          <t>cameraCenterAt: 400,600</t>
+          <t>cameraCenterAt: memory.homeX,self.resource.cameraY</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
@@ -5400,17 +5400,17 @@
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>deltaX,deltaY</t>
+          <t>runtimeDeltaX,runtimeDeltaY</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">
         <is>
-          <t>Moves the local owning player's camera center by a world-space offset.</t>
+          <t>Moves the local owning player's camera by a runtime-evaluated world-space offset.</t>
         </is>
       </c>
       <c r="E15" s="28" t="inlineStr">
         <is>
-          <t>cameraCenterBy: 80,-40</t>
+          <t>cameraCenterBy: cos(self.dir)*memory.distance,sin(self.dir)*memory.distance</t>
         </is>
       </c>
       <c r="F15" s="26" t="inlineStr">
@@ -5442,17 +5442,17 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>self|target|actionTarget[,offsetX,offsetY]</t>
+          <t>self|target|actionTarget[,runtimeOffsetX,runtimeOffsetY]</t>
         </is>
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
-          <t>Centers the camera on the acting unit, unit target, or action target point with an optional offset.</t>
+          <t>Centers the camera on a contextual target with optional runtime-evaluated offsets.</t>
         </is>
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>cameraCenterOn: actionTarget,0,-60</t>
+          <t>cameraCenterOn: actionTarget,memory.offsetX,clamp(self.hp,0,100)</t>
         </is>
       </c>
       <c r="F16" s="20" t="inlineStr">
@@ -5484,17 +5484,17 @@
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>positive float</t>
+          <t>positive runtime number</t>
         </is>
       </c>
       <c r="D17" s="28" t="inlineStr">
         <is>
-          <t>Sets the local owning player's native smoothed camera zoom target.</t>
+          <t>Sets the native smoothed camera zoom target from a runtime expression.</t>
         </is>
       </c>
       <c r="E17" s="28" t="inlineStr">
         <is>
-          <t>cameraTargetZoom: 1.25</t>
+          <t>cameraTargetZoom: clamp(memory.zoom,0.5,3)</t>
         </is>
       </c>
       <c r="F17" s="26" t="inlineStr">
@@ -5526,17 +5526,17 @@
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>runtime LogicBoolean</t>
         </is>
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Clears native camera scroll momentum when the action executes.</t>
+          <t>Clears native camera momentum when the runtime condition is true.</t>
         </is>
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>cameraStopMovement: true</t>
+          <t>cameraStopMovement: memory.lockCamera</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -6636,17 +6636,17 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>runtime LogicBoolean</t>
         </is>
       </c>
       <c r="D47" s="28" t="inlineStr">
         <is>
-          <t>Re-evaluates geometry and anchor while a persistent fog source is active.</t>
+          <t>Re-evaluates geometry and anchor while its runtime condition is true; otherwise uses the initial snapshot.</t>
         </is>
       </c>
       <c r="E47" s="28" t="inlineStr">
         <is>
-          <t>follow: true</t>
+          <t>follow: memory.trackingEnabled</t>
         </is>
       </c>
       <c r="F47" s="26" t="inlineStr">
@@ -13724,7 +13724,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>0.1.0</t>
@@ -13737,17 +13737,17 @@
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>runtime LogicBoolean</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>允许过量伤害使此自定义单位的生命值降到零以下，而不是夹到零。</t>
+          <t>当运行时条件为真时，允许过量伤害使此自定义单位的生命值降到零以下。</t>
         </is>
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>allowNegativeHp: true</t>
+          <t>allowNegativeHp: memory.berserk or self.resource.rage &gt; 0</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
@@ -13851,17 +13851,17 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>worldX,worldY</t>
+          <t>runtimeNumberX,runtimeNumberY</t>
         </is>
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>将本机单位所属玩家的视角中心移动到绝对世界坐标。</t>
+          <t>将本机玩家视角居中到运行时求值的绝对世界坐标。</t>
         </is>
       </c>
       <c r="E14" s="22" t="inlineStr">
         <is>
-          <t>cameraCenterAt: 400,600</t>
+          <t>cameraCenterAt: memory.homeX,self.resource.cameraY</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
@@ -13880,7 +13880,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
           <t>0.1.0</t>
@@ -13893,17 +13893,17 @@
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>deltaX,deltaY</t>
+          <t>runtimeDeltaX,runtimeDeltaY</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">
         <is>
-          <t>按照世界坐标偏移量移动本机单位所属玩家的视角中心。</t>
+          <t>按运行时求值的世界坐标偏移量移动本机玩家视角。</t>
         </is>
       </c>
       <c r="E15" s="28" t="inlineStr">
         <is>
-          <t>cameraCenterBy: 80,-40</t>
+          <t>cameraCenterBy: cos(self.dir)*memory.distance,sin(self.dir)*memory.distance</t>
         </is>
       </c>
       <c r="F15" s="26" t="inlineStr">
@@ -13922,7 +13922,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
           <t>0.1.0</t>
@@ -13935,17 +13935,17 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>self|target|actionTarget[,offsetX,offsetY]</t>
+          <t>self|target|actionTarget[,runtimeOffsetX,runtimeOffsetY]</t>
         </is>
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
-          <t>将视角居中到动作单位、目标单位或动作目标点，并可附加坐标偏移。</t>
+          <t>将视角居中到上下文目标，并可使用运行时求值的坐标偏移。</t>
         </is>
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>cameraCenterOn: actionTarget,0,-60</t>
+          <t>cameraCenterOn: actionTarget,memory.offsetX,clamp(self.hp,0,100)</t>
         </is>
       </c>
       <c r="F16" s="20" t="inlineStr">
@@ -13977,17 +13977,17 @@
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>positive float</t>
+          <t>positive runtime number</t>
         </is>
       </c>
       <c r="D17" s="28" t="inlineStr">
         <is>
-          <t>设置本机单位所属玩家的原版平滑视角缩放目标。</t>
+          <t>根据运行时表达式设置原版平滑视角缩放目标。</t>
         </is>
       </c>
       <c r="E17" s="28" t="inlineStr">
         <is>
-          <t>cameraTargetZoom: 1.25</t>
+          <t>cameraTargetZoom: clamp(memory.zoom,0.5,3)</t>
         </is>
       </c>
       <c r="F17" s="26" t="inlineStr">
@@ -14019,17 +14019,17 @@
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>runtime LogicBoolean</t>
         </is>
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>在动作执行时清除原版摄像机的滚动惯性。</t>
+          <t>当运行时条件为真时清除原版摄像机惯性。</t>
         </is>
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>cameraStopMovement: true</t>
+          <t>cameraStopMovement: memory.lockCamera</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -15129,17 +15129,17 @@
       </c>
       <c r="C47" s="26" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>runtime LogicBoolean</t>
         </is>
       </c>
       <c r="D47" s="28" t="inlineStr">
         <is>
-          <t>持续迷雾源生效时重新计算几何与锚点。</t>
+          <t>运行时条件为真时重新计算几何与锚点；否则使用初始快照。</t>
         </is>
       </c>
       <c r="E47" s="28" t="inlineStr">
         <is>
-          <t>follow: true</t>
+          <t>follow: memory.trackingEnabled</t>
         </is>
       </c>
       <c r="F47" s="26" t="inlineStr">

</xml_diff>

<commit_message>
Support native unit references in INI targets
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -1331,7 +1331,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="8096250"/>
+          <a:off x="14268450" y="8258175"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1372,7 +1372,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="14792325"/>
+          <a:off x="14268450" y="14954250"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1413,7 +1413,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="32546925"/>
+          <a:off x="14268450" y="32708850"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1454,7 +1454,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="35842575"/>
+          <a:off x="14268450" y="36214050"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1495,7 +1495,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="45605700"/>
+          <a:off x="14268450" y="45977175"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1536,7 +1536,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="51711225"/>
+          <a:off x="14268450" y="52082700"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1577,7 +1577,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="54292500"/>
+          <a:off x="14268450" y="54663975"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1618,7 +1618,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="58016775"/>
+          <a:off x="0" y="58388250"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1675,7 +1675,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="58016775"/>
+          <a:off x="3962400" y="58388250"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1732,7 +1732,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="58016775"/>
+          <a:off x="7924800" y="58388250"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1789,7 +1789,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="58016775"/>
+          <a:off x="11887200" y="58388250"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1846,7 +1846,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="58359675"/>
+          <a:off x="0" y="58731150"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1903,7 +1903,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="58359675"/>
+          <a:off x="3962400" y="58731150"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1960,7 +1960,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="58359675"/>
+          <a:off x="7924800" y="58731150"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2017,7 +2017,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="58359675"/>
+          <a:off x="11887200" y="58731150"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2074,7 +2074,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="58702575"/>
+          <a:off x="0" y="59074050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2131,7 +2131,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="58702575"/>
+          <a:off x="3962400" y="59074050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2188,7 +2188,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="58702575"/>
+          <a:off x="7924800" y="59074050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2245,7 +2245,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="58702575"/>
+          <a:off x="11887200" y="59074050"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2302,7 +2302,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="59045475"/>
+          <a:off x="0" y="59416950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2359,7 +2359,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="59045475"/>
+          <a:off x="3962400" y="59416950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2416,7 +2416,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="59045475"/>
+          <a:off x="7924800" y="59416950"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2473,7 +2473,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="59578875"/>
+          <a:off x="14268450" y="59950350"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2514,7 +2514,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="64512825"/>
+          <a:off x="14268450" y="64884300"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2555,7 +2555,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="69494400"/>
+          <a:off x="14268450" y="69865875"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2596,7 +2596,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="74475975"/>
+          <a:off x="14268450" y="74847450"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2637,7 +2637,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="78228825"/>
+          <a:off x="14268450" y="78600300"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2678,7 +2678,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="80752950"/>
+          <a:off x="14268450" y="81124425"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2719,7 +2719,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="84867750"/>
+          <a:off x="14268450" y="85239225"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2760,7 +2760,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="87487125"/>
+          <a:off x="14268450" y="87858600"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2801,7 +2801,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="91649550"/>
+          <a:off x="14268450" y="92021025"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2842,7 +2842,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="95402400"/>
+          <a:off x="14268450" y="95773875"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2883,7 +2883,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="98288475"/>
+          <a:off x="14268450" y="98659950"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2924,7 +2924,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="101993700"/>
+          <a:off x="14268450" y="102365175"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2965,7 +2965,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="105698925"/>
+          <a:off x="14268450" y="106070400"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3006,7 +3006,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="109404150"/>
+          <a:off x="14268450" y="109775625"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3047,7 +3047,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="113061750"/>
+          <a:off x="14268450" y="113433225"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3852,7 +3852,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="33794700"/>
+          <a:off x="14268450" y="33842325"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3893,7 +3893,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="43510200"/>
+          <a:off x="14268450" y="43557825"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3934,7 +3934,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="48977550"/>
+          <a:off x="14268450" y="49025175"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3975,7 +3975,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="51234975"/>
+          <a:off x="14268450" y="51282600"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4016,7 +4016,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="54702075"/>
+          <a:off x="0" y="54749700"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4073,7 +4073,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="54702075"/>
+          <a:off x="3962400" y="54749700"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4130,7 +4130,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="54702075"/>
+          <a:off x="7924800" y="54749700"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4187,7 +4187,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="54702075"/>
+          <a:off x="11887200" y="54749700"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4244,7 +4244,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="55044975"/>
+          <a:off x="0" y="55092600"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4301,7 +4301,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="55044975"/>
+          <a:off x="3962400" y="55092600"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4358,7 +4358,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="55044975"/>
+          <a:off x="7924800" y="55092600"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4415,7 +4415,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="55044975"/>
+          <a:off x="11887200" y="55092600"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4472,7 +4472,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="55387875"/>
+          <a:off x="0" y="55435500"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4529,7 +4529,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="55387875"/>
+          <a:off x="3962400" y="55435500"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4586,7 +4586,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="55387875"/>
+          <a:off x="7924800" y="55435500"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4643,7 +4643,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11887200" y="55387875"/>
+          <a:off x="11887200" y="55435500"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4700,7 +4700,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="55730775"/>
+          <a:off x="0" y="55778400"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4757,7 +4757,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3962400" y="55730775"/>
+          <a:off x="3962400" y="55778400"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4814,7 +4814,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="55730775"/>
+          <a:off x="7924800" y="55778400"/>
           <a:ext cx="3962400" cy="342900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4871,7 +4871,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="56264175"/>
+          <a:off x="14268450" y="56311800"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4912,7 +4912,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="60912375"/>
+          <a:off x="14268450" y="60960000"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4953,7 +4953,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="65703450"/>
+          <a:off x="14268450" y="65751075"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4994,7 +4994,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="70494525"/>
+          <a:off x="14268450" y="70542150"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5035,7 +5035,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="74199750"/>
+          <a:off x="14268450" y="74247375"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5076,7 +5076,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="76676250"/>
+          <a:off x="14268450" y="76723875"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5117,7 +5117,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="80600550"/>
+          <a:off x="14268450" y="80648175"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5158,7 +5158,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="83124675"/>
+          <a:off x="14268450" y="83172300"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5199,7 +5199,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="87096600"/>
+          <a:off x="14268450" y="87144225"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5240,7 +5240,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="90658950"/>
+          <a:off x="14268450" y="90706575"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5281,7 +5281,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="93497400"/>
+          <a:off x="14268450" y="93545025"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5322,7 +5322,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="97059750"/>
+          <a:off x="14268450" y="97107375"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5363,7 +5363,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="100622100"/>
+          <a:off x="14268450" y="100669725"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5404,7 +5404,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="104184450"/>
+          <a:off x="14268450" y="104232075"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5445,7 +5445,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14268450" y="107746800"/>
+          <a:off x="14268450" y="107794425"/>
           <a:ext cx="1581150" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6313,7 +6313,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
           <t>0.1.0</t>
@@ -6326,17 +6326,17 @@
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>self|target|actionTarget[,runtimeOffsetX,runtimeOffsetY]</t>
+          <t>(native UnitReference|actionTarget)[,optionalWorldOffsetX,optionalWorldOffsetY]</t>
         </is>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>Centers the camera on a contextual target with optional runtime-evaluated offsets.</t>
+          <t>Centers the camera on any native UnitReference or the contextual actionTarget point; the trailing world-axis X/Y offsets are optional together and default to zero.</t>
         </is>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>cameraCenterOn: actionTarget,memory.offsetX,clamp(self.hp,0,100)</t>
+          <t>cameraCenterOn: self.getOffsetRelative(x=20,y=100)</t>
         </is>
       </c>
       <c r="F17" s="24" t="inlineStr">
@@ -9259,7 +9259,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="28" customHeight="1">
+    <row r="91" ht="45" customHeight="1">
       <c r="A91" s="30" t="inlineStr">
         <is>
           <t>0.2.0</t>
@@ -9272,17 +9272,17 @@
       </c>
       <c r="C91" s="30" t="inlineStr">
         <is>
-          <t>self|target|actionTarget</t>
+          <t>native UnitReference|actionTarget</t>
         </is>
       </c>
       <c r="D91" s="32" t="inlineStr">
         <is>
-          <t>Selects the world-space anchor for the geometry.</t>
+          <t>Selects a world-space anchor from any native UnitReference or the contextual actionTarget point; follow=true reevaluates it.</t>
         </is>
       </c>
       <c r="E91" s="32" t="inlineStr">
         <is>
-          <t>anchor: actionTarget</t>
+          <t>anchor: self.customTarget1</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">
@@ -17703,17 +17703,17 @@
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>self|target|actionTarget[,runtimeOffsetX,runtimeOffsetY]</t>
+          <t>(native UnitReference|actionTarget)[,optionalWorldOffsetX,optionalWorldOffsetY]</t>
         </is>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>将视角居中到上下文目标，并可使用运行时求值的坐标偏移。</t>
+          <t>将视角居中到任意原版 UnitReference 或上下文 actionTarget 点；尾部世界轴 X/Y 偏移整体选填且默认均为零。</t>
         </is>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>cameraCenterOn: actionTarget,memory.offsetX,clamp(self.hp,0,100)</t>
+          <t>cameraCenterOn: self.getOffsetRelative(x=20,y=100)</t>
         </is>
       </c>
       <c r="F17" s="24" t="inlineStr">
@@ -20636,7 +20636,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="28" customHeight="1">
+    <row r="91" ht="32" customHeight="1">
       <c r="A91" s="30" t="inlineStr">
         <is>
           <t>0.2.0</t>
@@ -20649,17 +20649,17 @@
       </c>
       <c r="C91" s="30" t="inlineStr">
         <is>
-          <t>self|target|actionTarget</t>
+          <t>native UnitReference|actionTarget</t>
         </is>
       </c>
       <c r="D91" s="32" t="inlineStr">
         <is>
-          <t>选择几何遮罩的世界坐标锚点。</t>
+          <t>从任意原版 UnitReference 或上下文 actionTarget 点选择世界坐标锚点；follow=true 时会重新求值。</t>
         </is>
       </c>
       <c r="E91" s="32" t="inlineStr">
         <is>
-          <t>anchor: actionTarget</t>
+          <t>anchor: self.customTarget1</t>
         </is>
       </c>
       <c r="F91" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Refresh INI Essentials reference workbook
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -651,13 +651,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -669,7 +669,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1047750" y="2971800"/>
+          <a:off x="1047750" y="4000500"/>
           <a:ext cx="13220700" cy="400050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -692,13 +692,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -710,7 +710,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1047750" y="3371850"/>
+          <a:off x="1047750" y="4400550"/>
           <a:ext cx="13220700" cy="400050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7335,7 +7335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7351,7 +7351,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INI Essentials Unit Modding Reference</t>
+          <t>INI Essentials v0.2.0 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -7365,7 +7365,7 @@
     <row r="3" ht="27" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated from fields.csv and event-data.csv. Do not edit this workbook as the source.</t>
+          <t>Current mod version / 当前模组版本: 0.2.0</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -7379,7 +7379,7 @@
     <row r="4" ht="27" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>本表由 fields.csv 和 event-data.csv 自动生成，请勿把工作簿作为源文件直接修改。</t>
+          <t>Catalog Revision records feature-development batches; it is not the minimum installable mod version.</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -7393,7 +7393,7 @@
     <row r="5" ht="27" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Native keys with native-valid values stay on the native parser path.</t>
+          <t>目录修订记录功能开发批次，并不表示所需安装的最低模组版本。</t>
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
@@ -7407,7 +7407,7 @@
     <row r="6" ht="27" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>原版字段使用原版合法值时，始终保留原版解析路径。</t>
+          <t>Generated from fields.csv and event-data.csv. Do not edit this workbook as the source.</t>
         </is>
       </c>
       <c r="B6" s="3" t="n"/>
@@ -7421,7 +7421,7 @@
     <row r="7" ht="27" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Extensions activate only for a documented new key, value range, format, or event-data name.</t>
+          <t>本表由 fields.csv 和 event-data.csv 自动生成，请勿把工作簿作为源文件直接修改。</t>
         </is>
       </c>
       <c r="B7" s="2" t="n"/>
@@ -7435,7 +7435,7 @@
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>只有代码表明确记录的新字段、新取值范围、新格式或事件数据名才会激活扩展。</t>
+          <t>Native keys with native-valid values stay on the native parser path.</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
@@ -7446,41 +7446,86 @@
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
     </row>
-    <row r="10" ht="31" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
+    <row r="9" ht="27" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>原版字段使用原版合法值时，始终保留原版解析路径。</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="27" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Extensions activate only for a documented new key, value range, format, or event-data name.</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="27" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>只有代码表明确记录的新字段、新取值范围、新格式或事件数据名才会激活扩展。</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+    </row>
+    <row r="13" ht="31" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Open English reference / 打开英文代码表</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="31" customHeight="1">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="31" customHeight="1">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>打开简体中文代码表 / Open Chinese reference</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A9:H9"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="B10:G10"/>
     <mergeCell ref="A7:H7"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="B13:G13"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A6:H6"/>
-    <mergeCell ref="B11:G11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rIdRFNavigation"/>
@@ -7509,7 +7554,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials Unit Modding Reference</t>
+          <t>INI Essentials v0.2.0 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>
@@ -7635,7 +7680,7 @@
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
@@ -7665,7 +7710,7 @@
     <row r="10" ht="31" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B10" s="24" t="inlineStr">
@@ -7749,7 +7794,7 @@
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B13" s="28" t="inlineStr">
@@ -7779,7 +7824,7 @@
     <row r="14" ht="31" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -8283,7 +8328,7 @@
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="34" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B27" s="34" t="inlineStr">
@@ -8313,7 +8358,7 @@
     <row r="28" ht="31" customHeight="1">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B28" s="36" t="inlineStr">
@@ -8985,7 +9030,7 @@
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="37" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B45" s="37" t="inlineStr">
@@ -9015,7 +9060,7 @@
     <row r="46" ht="31" customHeight="1">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B46" s="39" t="inlineStr">
@@ -11661,7 +11706,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="40" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B110" s="40" t="inlineStr">
@@ -11691,7 +11736,7 @@
     <row r="111" ht="31" customHeight="1">
       <c r="A111" s="42" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B111" s="42" t="inlineStr">
@@ -12363,7 +12408,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="43" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B128" s="43" t="inlineStr">
@@ -12393,7 +12438,7 @@
     <row r="129" ht="31" customHeight="1">
       <c r="A129" s="45" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B129" s="45" t="inlineStr">
@@ -12687,7 +12732,7 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="46" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B137" s="46" t="inlineStr">
@@ -12717,7 +12762,7 @@
     <row r="138" ht="31" customHeight="1">
       <c r="A138" s="48" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B138" s="48" t="inlineStr">
@@ -14019,7 +14064,7 @@
     <row r="170" ht="34" customHeight="1">
       <c r="A170" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B170" s="49" t="inlineStr">
@@ -14049,7 +14094,7 @@
     <row r="171" ht="31" customHeight="1">
       <c r="A171" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B171" s="51" t="inlineStr">
@@ -14595,7 +14640,7 @@
     <row r="185" ht="34" customHeight="1">
       <c r="A185" s="52" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B185" s="52" t="inlineStr">
@@ -14625,7 +14670,7 @@
     <row r="186" ht="31" customHeight="1">
       <c r="A186" s="54" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B186" s="54" t="inlineStr">
@@ -14793,7 +14838,7 @@
     <row r="191" ht="34" customHeight="1">
       <c r="A191" s="55" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B191" s="55" t="inlineStr">
@@ -14823,7 +14868,7 @@
     <row r="192" ht="31" customHeight="1">
       <c r="A192" s="57" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B192" s="57" t="inlineStr">
@@ -15297,7 +15342,7 @@
     <row r="207" ht="34" customHeight="1">
       <c r="A207" s="58" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B207" s="58" t="inlineStr">
@@ -15327,7 +15372,7 @@
     <row r="208" ht="31" customHeight="1">
       <c r="A208" s="60" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B208" s="60" t="inlineStr">
@@ -15537,7 +15582,7 @@
     <row r="214" ht="34" customHeight="1">
       <c r="A214" s="58" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B214" s="58" t="inlineStr">
@@ -15567,7 +15612,7 @@
     <row r="215" ht="31" customHeight="1">
       <c r="A215" s="60" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B215" s="60" t="inlineStr">
@@ -16113,7 +16158,7 @@
     <row r="229" ht="34" customHeight="1">
       <c r="A229" s="58" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B229" s="58" t="inlineStr">
@@ -16143,7 +16188,7 @@
     <row r="230" ht="31" customHeight="1">
       <c r="A230" s="60" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B230" s="60" t="inlineStr">
@@ -16689,7 +16734,7 @@
     <row r="244" ht="34" customHeight="1">
       <c r="A244" s="58" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B244" s="58" t="inlineStr">
@@ -16719,7 +16764,7 @@
     <row r="245" ht="31" customHeight="1">
       <c r="A245" s="60" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B245" s="60" t="inlineStr">
@@ -16803,7 +16848,7 @@
     <row r="248" ht="34" customHeight="1">
       <c r="A248" s="58" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B248" s="58" t="inlineStr">
@@ -16833,7 +16878,7 @@
     <row r="249" ht="31" customHeight="1">
       <c r="A249" s="60" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B249" s="60" t="inlineStr">
@@ -16917,7 +16962,7 @@
     <row r="252" ht="34" customHeight="1">
       <c r="A252" s="58" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B252" s="58" t="inlineStr">
@@ -16947,7 +16992,7 @@
     <row r="253" ht="31" customHeight="1">
       <c r="A253" s="60" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B253" s="60" t="inlineStr">
@@ -18081,7 +18126,7 @@
     <row r="285" ht="34" customHeight="1">
       <c r="A285" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B285" s="49" t="inlineStr">
@@ -18111,7 +18156,7 @@
     <row r="286" ht="31" customHeight="1">
       <c r="A286" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B286" s="51" t="inlineStr">
@@ -18573,7 +18618,7 @@
     <row r="298" ht="34" customHeight="1">
       <c r="A298" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B298" s="49" t="inlineStr">
@@ -18603,7 +18648,7 @@
     <row r="299" ht="31" customHeight="1">
       <c r="A299" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B299" s="51" t="inlineStr">
@@ -19065,7 +19110,7 @@
     <row r="311" ht="34" customHeight="1">
       <c r="A311" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B311" s="49" t="inlineStr">
@@ -19095,7 +19140,7 @@
     <row r="312" ht="31" customHeight="1">
       <c r="A312" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B312" s="51" t="inlineStr">
@@ -19557,7 +19602,7 @@
     <row r="324" ht="34" customHeight="1">
       <c r="A324" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B324" s="49" t="inlineStr">
@@ -19587,7 +19632,7 @@
     <row r="325" ht="31" customHeight="1">
       <c r="A325" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B325" s="51" t="inlineStr">
@@ -19923,7 +19968,7 @@
     <row r="334" ht="34" customHeight="1">
       <c r="A334" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B334" s="49" t="inlineStr">
@@ -19953,7 +19998,7 @@
     <row r="335" ht="31" customHeight="1">
       <c r="A335" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B335" s="51" t="inlineStr">
@@ -20163,7 +20208,7 @@
     <row r="341" ht="34" customHeight="1">
       <c r="A341" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B341" s="49" t="inlineStr">
@@ -20193,7 +20238,7 @@
     <row r="342" ht="31" customHeight="1">
       <c r="A342" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B342" s="51" t="inlineStr">
@@ -20571,7 +20616,7 @@
     <row r="352" ht="34" customHeight="1">
       <c r="A352" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B352" s="49" t="inlineStr">
@@ -20601,7 +20646,7 @@
     <row r="353" ht="31" customHeight="1">
       <c r="A353" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B353" s="51" t="inlineStr">
@@ -20811,7 +20856,7 @@
     <row r="359" ht="34" customHeight="1">
       <c r="A359" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B359" s="49" t="inlineStr">
@@ -20841,7 +20886,7 @@
     <row r="360" ht="31" customHeight="1">
       <c r="A360" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B360" s="51" t="inlineStr">
@@ -21219,7 +21264,7 @@
     <row r="370" ht="34" customHeight="1">
       <c r="A370" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B370" s="49" t="inlineStr">
@@ -21249,7 +21294,7 @@
     <row r="371" ht="31" customHeight="1">
       <c r="A371" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B371" s="51" t="inlineStr">
@@ -21585,7 +21630,7 @@
     <row r="380" ht="34" customHeight="1">
       <c r="A380" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B380" s="49" t="inlineStr">
@@ -21615,7 +21660,7 @@
     <row r="381" ht="31" customHeight="1">
       <c r="A381" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B381" s="51" t="inlineStr">
@@ -21867,7 +21912,7 @@
     <row r="388" ht="34" customHeight="1">
       <c r="A388" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B388" s="49" t="inlineStr">
@@ -21897,7 +21942,7 @@
     <row r="389" ht="31" customHeight="1">
       <c r="A389" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B389" s="51" t="inlineStr">
@@ -22233,7 +22278,7 @@
     <row r="398" ht="34" customHeight="1">
       <c r="A398" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B398" s="49" t="inlineStr">
@@ -22263,7 +22308,7 @@
     <row r="399" ht="31" customHeight="1">
       <c r="A399" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B399" s="51" t="inlineStr">
@@ -22599,7 +22644,7 @@
     <row r="408" ht="34" customHeight="1">
       <c r="A408" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B408" s="49" t="inlineStr">
@@ -22629,7 +22674,7 @@
     <row r="409" ht="31" customHeight="1">
       <c r="A409" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B409" s="51" t="inlineStr">
@@ -22965,7 +23010,7 @@
     <row r="418" ht="34" customHeight="1">
       <c r="A418" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B418" s="49" t="inlineStr">
@@ -22995,7 +23040,7 @@
     <row r="419" ht="31" customHeight="1">
       <c r="A419" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B419" s="51" t="inlineStr">
@@ -23331,7 +23376,7 @@
     <row r="428" ht="34" customHeight="1">
       <c r="A428" s="49" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="B428" s="49" t="inlineStr">
@@ -23361,7 +23406,7 @@
     <row r="429" ht="31" customHeight="1">
       <c r="A429" s="51" t="inlineStr">
         <is>
-          <t>Version Added</t>
+          <t>Catalog Revision</t>
         </is>
       </c>
       <c r="B429" s="51" t="inlineStr">
@@ -23796,7 +23841,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials 单位模组代码表</t>
+          <t>INI Essentials v0.2.0 单位模组代码表</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>
@@ -23922,7 +23967,7 @@
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
@@ -23952,7 +23997,7 @@
     <row r="10" ht="31" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B10" s="24" t="inlineStr">
@@ -24036,7 +24081,7 @@
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B13" s="28" t="inlineStr">
@@ -24066,7 +24111,7 @@
     <row r="14" ht="31" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -24570,7 +24615,7 @@
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="34" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B27" s="34" t="inlineStr">
@@ -24600,7 +24645,7 @@
     <row r="28" ht="31" customHeight="1">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B28" s="36" t="inlineStr">
@@ -25272,7 +25317,7 @@
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="37" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B45" s="37" t="inlineStr">
@@ -25302,7 +25347,7 @@
     <row r="46" ht="31" customHeight="1">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B46" s="39" t="inlineStr">
@@ -27948,7 +27993,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="40" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B110" s="40" t="inlineStr">
@@ -27978,7 +28023,7 @@
     <row r="111" ht="31" customHeight="1">
       <c r="A111" s="42" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B111" s="42" t="inlineStr">
@@ -28650,7 +28695,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="43" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B128" s="43" t="inlineStr">
@@ -28680,7 +28725,7 @@
     <row r="129" ht="31" customHeight="1">
       <c r="A129" s="45" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B129" s="45" t="inlineStr">
@@ -28974,7 +29019,7 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="46" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B137" s="46" t="inlineStr">
@@ -29004,7 +29049,7 @@
     <row r="138" ht="31" customHeight="1">
       <c r="A138" s="48" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B138" s="48" t="inlineStr">
@@ -30306,7 +30351,7 @@
     <row r="170" ht="34" customHeight="1">
       <c r="A170" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B170" s="49" t="inlineStr">
@@ -30336,7 +30381,7 @@
     <row r="171" ht="31" customHeight="1">
       <c r="A171" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B171" s="51" t="inlineStr">
@@ -30882,7 +30927,7 @@
     <row r="185" ht="34" customHeight="1">
       <c r="A185" s="52" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B185" s="52" t="inlineStr">
@@ -30912,7 +30957,7 @@
     <row r="186" ht="31" customHeight="1">
       <c r="A186" s="54" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B186" s="54" t="inlineStr">
@@ -31080,7 +31125,7 @@
     <row r="191" ht="34" customHeight="1">
       <c r="A191" s="55" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B191" s="55" t="inlineStr">
@@ -31110,7 +31155,7 @@
     <row r="192" ht="31" customHeight="1">
       <c r="A192" s="57" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B192" s="57" t="inlineStr">
@@ -31584,7 +31629,7 @@
     <row r="207" ht="34" customHeight="1">
       <c r="A207" s="58" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B207" s="58" t="inlineStr">
@@ -31614,7 +31659,7 @@
     <row r="208" ht="31" customHeight="1">
       <c r="A208" s="60" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B208" s="60" t="inlineStr">
@@ -31824,7 +31869,7 @@
     <row r="214" ht="34" customHeight="1">
       <c r="A214" s="58" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B214" s="58" t="inlineStr">
@@ -31854,7 +31899,7 @@
     <row r="215" ht="31" customHeight="1">
       <c r="A215" s="60" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B215" s="60" t="inlineStr">
@@ -32400,7 +32445,7 @@
     <row r="229" ht="34" customHeight="1">
       <c r="A229" s="58" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B229" s="58" t="inlineStr">
@@ -32430,7 +32475,7 @@
     <row r="230" ht="31" customHeight="1">
       <c r="A230" s="60" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B230" s="60" t="inlineStr">
@@ -32976,7 +33021,7 @@
     <row r="244" ht="34" customHeight="1">
       <c r="A244" s="58" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B244" s="58" t="inlineStr">
@@ -33006,7 +33051,7 @@
     <row r="245" ht="31" customHeight="1">
       <c r="A245" s="60" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B245" s="60" t="inlineStr">
@@ -33090,7 +33135,7 @@
     <row r="248" ht="34" customHeight="1">
       <c r="A248" s="58" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B248" s="58" t="inlineStr">
@@ -33120,7 +33165,7 @@
     <row r="249" ht="31" customHeight="1">
       <c r="A249" s="60" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B249" s="60" t="inlineStr">
@@ -33204,7 +33249,7 @@
     <row r="252" ht="34" customHeight="1">
       <c r="A252" s="58" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B252" s="58" t="inlineStr">
@@ -33234,7 +33279,7 @@
     <row r="253" ht="31" customHeight="1">
       <c r="A253" s="60" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B253" s="60" t="inlineStr">
@@ -34368,7 +34413,7 @@
     <row r="285" ht="34" customHeight="1">
       <c r="A285" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B285" s="49" t="inlineStr">
@@ -34398,7 +34443,7 @@
     <row r="286" ht="31" customHeight="1">
       <c r="A286" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B286" s="51" t="inlineStr">
@@ -34860,7 +34905,7 @@
     <row r="298" ht="34" customHeight="1">
       <c r="A298" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B298" s="49" t="inlineStr">
@@ -34890,7 +34935,7 @@
     <row r="299" ht="31" customHeight="1">
       <c r="A299" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B299" s="51" t="inlineStr">
@@ -35352,7 +35397,7 @@
     <row r="311" ht="34" customHeight="1">
       <c r="A311" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B311" s="49" t="inlineStr">
@@ -35382,7 +35427,7 @@
     <row r="312" ht="31" customHeight="1">
       <c r="A312" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B312" s="51" t="inlineStr">
@@ -35844,7 +35889,7 @@
     <row r="324" ht="34" customHeight="1">
       <c r="A324" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B324" s="49" t="inlineStr">
@@ -35874,7 +35919,7 @@
     <row r="325" ht="31" customHeight="1">
       <c r="A325" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B325" s="51" t="inlineStr">
@@ -36210,7 +36255,7 @@
     <row r="334" ht="34" customHeight="1">
       <c r="A334" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B334" s="49" t="inlineStr">
@@ -36240,7 +36285,7 @@
     <row r="335" ht="31" customHeight="1">
       <c r="A335" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B335" s="51" t="inlineStr">
@@ -36450,7 +36495,7 @@
     <row r="341" ht="34" customHeight="1">
       <c r="A341" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B341" s="49" t="inlineStr">
@@ -36480,7 +36525,7 @@
     <row r="342" ht="31" customHeight="1">
       <c r="A342" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B342" s="51" t="inlineStr">
@@ -36858,7 +36903,7 @@
     <row r="352" ht="34" customHeight="1">
       <c r="A352" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B352" s="49" t="inlineStr">
@@ -36888,7 +36933,7 @@
     <row r="353" ht="31" customHeight="1">
       <c r="A353" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B353" s="51" t="inlineStr">
@@ -37098,7 +37143,7 @@
     <row r="359" ht="34" customHeight="1">
       <c r="A359" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B359" s="49" t="inlineStr">
@@ -37128,7 +37173,7 @@
     <row r="360" ht="31" customHeight="1">
       <c r="A360" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B360" s="51" t="inlineStr">
@@ -37506,7 +37551,7 @@
     <row r="370" ht="34" customHeight="1">
       <c r="A370" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B370" s="49" t="inlineStr">
@@ -37536,7 +37581,7 @@
     <row r="371" ht="31" customHeight="1">
       <c r="A371" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B371" s="51" t="inlineStr">
@@ -37872,7 +37917,7 @@
     <row r="380" ht="34" customHeight="1">
       <c r="A380" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B380" s="49" t="inlineStr">
@@ -37902,7 +37947,7 @@
     <row r="381" ht="31" customHeight="1">
       <c r="A381" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B381" s="51" t="inlineStr">
@@ -38154,7 +38199,7 @@
     <row r="388" ht="34" customHeight="1">
       <c r="A388" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B388" s="49" t="inlineStr">
@@ -38184,7 +38229,7 @@
     <row r="389" ht="31" customHeight="1">
       <c r="A389" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B389" s="51" t="inlineStr">
@@ -38520,7 +38565,7 @@
     <row r="398" ht="34" customHeight="1">
       <c r="A398" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B398" s="49" t="inlineStr">
@@ -38550,7 +38595,7 @@
     <row r="399" ht="31" customHeight="1">
       <c r="A399" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B399" s="51" t="inlineStr">
@@ -38886,7 +38931,7 @@
     <row r="408" ht="34" customHeight="1">
       <c r="A408" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B408" s="49" t="inlineStr">
@@ -38916,7 +38961,7 @@
     <row r="409" ht="31" customHeight="1">
       <c r="A409" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B409" s="51" t="inlineStr">
@@ -39252,7 +39297,7 @@
     <row r="418" ht="34" customHeight="1">
       <c r="A418" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B418" s="49" t="inlineStr">
@@ -39282,7 +39327,7 @@
     <row r="419" ht="31" customHeight="1">
       <c r="A419" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B419" s="51" t="inlineStr">
@@ -39618,7 +39663,7 @@
     <row r="428" ht="34" customHeight="1">
       <c r="A428" s="49" t="inlineStr">
         <is>
-          <t>版本</t>
+          <t>目录</t>
         </is>
       </c>
       <c r="B428" s="49" t="inlineStr">
@@ -39648,7 +39693,7 @@
     <row r="429" ht="31" customHeight="1">
       <c r="A429" s="51" t="inlineStr">
         <is>
-          <t>加入版本</t>
+          <t>目录修订</t>
         </is>
       </c>
       <c r="B429" s="51" t="inlineStr">

</xml_diff>

<commit_message>
Prepare v0.3.0 release versions
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -7945,7 +7945,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INI Essentials v0.2.0 Unit Modding Reference</t>
+          <t>INI Essentials v0.2.1 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -7959,7 +7959,7 @@
     <row r="3" ht="27" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Current mod version / 当前模组版本: 0.2.0</t>
+          <t>Current mod version / 当前模组版本: 0.2.1</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -8148,7 +8148,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials v0.2.0 Unit Modding Reference</t>
+          <t>INI Essentials v0.2.1 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>
@@ -24677,7 +24677,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials v0.2.0 单位模组代码表</t>
+          <t>INI Essentials v0.2.1 单位模组代码表</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>

</xml_diff>

<commit_message>
Prepare Rusted Fabric 0.4.0 release
Advertise the official QQ group in both launchers, bump changed component versions and API constraints, and refresh release documentation.
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -7945,7 +7945,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INI Essentials v0.2.1 Unit Modding Reference</t>
+          <t>INI Essentials v0.3.0 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -7959,7 +7959,7 @@
     <row r="3" ht="27" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Current mod version / 当前模组版本: 0.2.1</t>
+          <t>Current mod version / 当前模组版本: 0.3.0</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -8148,7 +8148,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials v0.2.1 Unit Modding Reference</t>
+          <t>INI Essentials v0.3.0 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>
@@ -24929,7 +24929,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials v0.2.1 单位模组代码表</t>
+          <t>INI Essentials v0.3.0 单位模组代码表</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>

</xml_diff>

<commit_message>
Prepare Rusted Fabric 0.4.2 release
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -36,6 +36,7 @@
     <definedName name="rf_en_custom_projectile_collision">'English'!$A$272</definedName>
     <definedName name="rf_en_custom_projectile_effect">'English'!$A$287</definedName>
     <definedName name="rf_en_custom_projectile_decal">'English'!$A$291</definedName>
+    <definedName name="rf_en_class_event_context">'English'!$A$295</definedName>
     <definedName name="rf_en_event_data">'English'!$A$295</definedName>
     <definedName name="rf_en_event_shortcuts">'English'!$A$296</definedName>
     <definedName name="rf_en_event_tookdamage">'English'!$A$302</definedName>
@@ -77,6 +78,7 @@
     <definedName name="rf_zh_custom_projectile_collision">'简体中文'!$A$272</definedName>
     <definedName name="rf_zh_custom_projectile_effect">'简体中文'!$A$287</definedName>
     <definedName name="rf_zh_custom_projectile_decal">'简体中文'!$A$291</definedName>
+    <definedName name="rf_zh_class_event_context">'简体中文'!$A$295</definedName>
     <definedName name="rf_zh_event_data">'简体中文'!$A$295</definedName>
     <definedName name="rf_zh_event_shortcuts">'简体中文'!$A$296</definedName>
     <definedName name="rf_zh_event_tookdamage">'简体中文'!$A$302</definedName>
@@ -207,11 +209,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1565C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
@@ -312,6 +309,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1565C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF0D47A1"/>
       </patternFill>
     </fill>
@@ -391,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -414,13 +416,16 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -447,9 +452,6 @@
     <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -458,7 +460,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -478,6 +480,15 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -551,25 +562,19 @@
     <xf numFmtId="0" fontId="3" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -749,7 +754,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>3714750</xdr:colOff>
+      <xdr:colOff>1066800</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -763,7 +768,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="857250"/>
-          <a:ext cx="7924800" cy="285750"/>
+          <a:ext cx="5276850" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -800,13 +805,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>3714750</xdr:colOff>
+      <xdr:colOff>1066800</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1771650</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -819,8 +824,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="857250"/>
-          <a:ext cx="7924800" cy="285750"/>
+          <a:off x="5276850" y="857250"/>
+          <a:ext cx="5286375" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -856,6 +861,63 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1771650</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="class_en_2">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10563225" y="857250"/>
+          <a:ext cx="5286375" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="00A6B8"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="A6A6A6"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="45720" tIns="0" rIns="45720" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:rPr>
+            <a:t>EventContext</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
@@ -869,8 +931,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="shortcut_en_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        <xdr:cNvPr id="4" name="shortcut_en_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -926,8 +988,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="shortcut_en_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        <xdr:cNvPr id="5" name="shortcut_en_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -983,8 +1045,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="shortcut_en_geometry">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        <xdr:cNvPr id="6" name="shortcut_en_geometry">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1040,8 +1102,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="shortcut_en_overlay">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        <xdr:cNvPr id="7" name="shortcut_en_overlay">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1097,8 +1159,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="shortcut_en_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        <xdr:cNvPr id="8" name="shortcut_en_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1154,8 +1216,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="shortcut_en_fog">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        <xdr:cNvPr id="9" name="shortcut_en_fog">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1211,8 +1273,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="shortcut_en_math">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        <xdr:cNvPr id="10" name="shortcut_en_math">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1268,8 +1330,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="shortcut_en_event">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+        <xdr:cNvPr id="11" name="shortcut_en_event">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1325,8 +1387,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="shortcut_en_projectile">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+        <xdr:cNvPr id="12" name="shortcut_en_projectile">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1382,8 +1444,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="shortcut_en_turret">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+        <xdr:cNvPr id="13" name="shortcut_en_turret">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1439,8 +1501,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="back_en_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+        <xdr:cNvPr id="14" name="back_en_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1480,8 +1542,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="back_en_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+        <xdr:cNvPr id="15" name="back_en_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1521,8 +1583,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="back_en_geometry">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+        <xdr:cNvPr id="16" name="back_en_geometry">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1562,8 +1624,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="back_en_overlay">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+        <xdr:cNvPr id="17" name="back_en_overlay">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1603,8 +1665,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="back_en_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+        <xdr:cNvPr id="18" name="back_en_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1644,8 +1706,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="back_en_fog">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+        <xdr:cNvPr id="19" name="back_en_fog">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1685,8 +1747,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="19" name="back_en_math">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
+        <xdr:cNvPr id="20" name="back_en_math">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1726,8 +1788,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="20" name="back_en_event">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
+        <xdr:cNvPr id="21" name="back_en_event">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1767,8 +1829,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="back_en_projectile">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
+        <xdr:cNvPr id="22" name="back_en_projectile">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1808,8 +1870,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="back_en_turret">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
+        <xdr:cNvPr id="23" name="back_en_turret">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1849,8 +1911,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="shortcut_en_custom_projectile_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
+        <xdr:cNvPr id="24" name="shortcut_en_custom_projectile_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1906,8 +1968,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="shortcut_en_custom_projectile_pattern">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
+        <xdr:cNvPr id="25" name="shortcut_en_custom_projectile_pattern">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -1963,8 +2025,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="shortcut_en_custom_projectile_motion">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
+        <xdr:cNvPr id="26" name="shortcut_en_custom_projectile_motion">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2020,8 +2082,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="shortcut_en_custom_projectile_lifecycle">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
+        <xdr:cNvPr id="27" name="shortcut_en_custom_projectile_lifecycle">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2077,8 +2139,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="shortcut_en_custom_projectile_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
+        <xdr:cNvPr id="28" name="shortcut_en_custom_projectile_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2134,8 +2196,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="shortcut_en_custom_projectile_runtime">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
+        <xdr:cNvPr id="29" name="shortcut_en_custom_projectile_runtime">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2191,8 +2253,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="shortcut_en_custom_projectile_collision">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
+        <xdr:cNvPr id="30" name="shortcut_en_custom_projectile_collision">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2248,8 +2310,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="shortcut_en_custom_projectile_effect">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
+        <xdr:cNvPr id="31" name="shortcut_en_custom_projectile_effect">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2305,8 +2367,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="shortcut_en_custom_projectile_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
+        <xdr:cNvPr id="32" name="shortcut_en_custom_projectile_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2362,8 +2424,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="32" name="back_en_custom_projectile_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
+        <xdr:cNvPr id="33" name="back_en_custom_projectile_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2403,8 +2465,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="33" name="back_en_custom_projectile_pattern">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33"/>
+        <xdr:cNvPr id="34" name="back_en_custom_projectile_pattern">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2444,8 +2506,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="34" name="back_en_custom_projectile_motion">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
+        <xdr:cNvPr id="35" name="back_en_custom_projectile_motion">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2485,8 +2547,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="35" name="back_en_custom_projectile_lifecycle">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35"/>
+        <xdr:cNvPr id="36" name="back_en_custom_projectile_lifecycle">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2526,8 +2588,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="36" name="back_en_custom_projectile_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
+        <xdr:cNvPr id="37" name="back_en_custom_projectile_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2567,8 +2629,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="37" name="back_en_custom_projectile_runtime">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
+        <xdr:cNvPr id="38" name="back_en_custom_projectile_runtime">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2608,8 +2670,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="38" name="back_en_custom_projectile_collision">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
+        <xdr:cNvPr id="39" name="back_en_custom_projectile_collision">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2649,8 +2711,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="39" name="back_en_custom_projectile_effect">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
+        <xdr:cNvPr id="40" name="back_en_custom_projectile_effect">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId40"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2690,8 +2752,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="40" name="back_en_custom_projectile_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId40"/>
+        <xdr:cNvPr id="41" name="back_en_custom_projectile_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2731,8 +2793,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="41" name="shortcut_en_event_tookdamage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41"/>
+        <xdr:cNvPr id="42" name="shortcut_en_event_tookdamage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId42"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2788,8 +2850,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="42" name="shortcut_en_event_queueitemadded">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId42"/>
+        <xdr:cNvPr id="43" name="shortcut_en_event_queueitemadded">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2845,8 +2907,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="43" name="shortcut_en_event_queueitemcancelled">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43"/>
+        <xdr:cNvPr id="44" name="shortcut_en_event_queueitemcancelled">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId44"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2902,8 +2964,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="44" name="shortcut_en_event_newwaypointgivenbyplayer">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId44"/>
+        <xdr:cNvPr id="45" name="shortcut_en_event_newwaypointgivenbyplayer">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -2959,8 +3021,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="45" name="shortcut_en_event_teamchanged">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45"/>
+        <xdr:cNvPr id="46" name="shortcut_en_event_teamchanged">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId46"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3016,8 +3078,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="46" name="shortcut_en_event_teleported">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId46"/>
+        <xdr:cNvPr id="47" name="shortcut_en_event_teleported">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3073,8 +3135,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="47" name="shortcut_en_event_attachmentremoved">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47"/>
+        <xdr:cNvPr id="48" name="shortcut_en_event_attachmentremoved">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId48"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3130,8 +3192,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="48" name="shortcut_en_event_killedanyunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId48"/>
+        <xdr:cNvPr id="49" name="shortcut_en_event_killedanyunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3187,8 +3249,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="49" name="shortcut_en_event_queuedunitfinished">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49"/>
+        <xdr:cNvPr id="50" name="shortcut_en_event_queuedunitfinished">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3244,8 +3306,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="50" name="shortcut_en_event_touchtargetsuccess">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
+        <xdr:cNvPr id="51" name="shortcut_en_event_touchtargetsuccess">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3301,8 +3363,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="51" name="shortcut_en_event_transportingnewunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
+        <xdr:cNvPr id="52" name="shortcut_en_event_transportingnewunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId52"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3358,8 +3420,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="52" name="shortcut_en_event_transportunloadedorremovedunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId52"/>
+        <xdr:cNvPr id="53" name="shortcut_en_event_transportunloadedorremovedunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3415,8 +3477,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="53" name="shortcut_en_event_enteredtransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
+        <xdr:cNvPr id="54" name="shortcut_en_event_enteredtransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId54"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3472,8 +3534,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="54" name="shortcut_en_event_lefttransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId54"/>
+        <xdr:cNvPr id="55" name="shortcut_en_event_lefttransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3529,8 +3591,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="55" name="shortcut_en_event_newmessage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
+        <xdr:cNvPr id="56" name="shortcut_en_event_newmessage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId56"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3586,8 +3648,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="56" name="back_en_event_tookdamage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId56"/>
+        <xdr:cNvPr id="57" name="back_en_event_tookdamage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3627,8 +3689,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="57" name="back_en_event_queueitemadded">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
+        <xdr:cNvPr id="58" name="back_en_event_queueitemadded">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId58"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3668,8 +3730,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="58" name="back_en_event_queueitemcancelled">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId58"/>
+        <xdr:cNvPr id="59" name="back_en_event_queueitemcancelled">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3709,8 +3771,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="59" name="back_en_event_newwaypointgivenbyplayer">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
+        <xdr:cNvPr id="60" name="back_en_event_newwaypointgivenbyplayer">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId60"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3750,8 +3812,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="60" name="back_en_event_teamchanged">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId60"/>
+        <xdr:cNvPr id="61" name="back_en_event_teamchanged">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId61"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3791,8 +3853,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="61" name="back_en_event_teleported">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId61"/>
+        <xdr:cNvPr id="62" name="back_en_event_teleported">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId62"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3832,8 +3894,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="62" name="back_en_event_attachmentremoved">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId62"/>
+        <xdr:cNvPr id="63" name="back_en_event_attachmentremoved">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3873,8 +3935,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="63" name="back_en_event_killedanyunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63"/>
+        <xdr:cNvPr id="64" name="back_en_event_killedanyunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId64"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3914,8 +3976,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="64" name="back_en_event_queuedunitfinished">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId64"/>
+        <xdr:cNvPr id="65" name="back_en_event_queuedunitfinished">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId65"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3955,8 +4017,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="65" name="back_en_event_touchtargetsuccess">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId65"/>
+        <xdr:cNvPr id="66" name="back_en_event_touchtargetsuccess">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -3996,8 +4058,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="66" name="back_en_event_transportingnewunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
+        <xdr:cNvPr id="67" name="back_en_event_transportingnewunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4037,8 +4099,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="67" name="back_en_event_transportunloadedorremovedunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
+        <xdr:cNvPr id="68" name="back_en_event_transportunloadedorremovedunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId68"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4078,8 +4140,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="68" name="back_en_event_enteredtransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId68"/>
+        <xdr:cNvPr id="69" name="back_en_event_enteredtransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4119,8 +4181,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="69" name="back_en_event_lefttransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
+        <xdr:cNvPr id="70" name="back_en_event_lefttransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4160,8 +4222,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="70" name="back_en_event_newmessage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
+        <xdr:cNvPr id="71" name="back_en_event_newmessage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4200,7 +4262,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>3714750</xdr:colOff>
+      <xdr:colOff>1066800</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -4214,7 +4276,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="857250"/>
-          <a:ext cx="7924800" cy="285750"/>
+          <a:ext cx="5276850" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4251,13 +4313,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>3714750</xdr:colOff>
+      <xdr:colOff>1066800</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1771650</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -4270,8 +4332,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="857250"/>
-          <a:ext cx="7924800" cy="285750"/>
+          <a:off x="5276850" y="857250"/>
+          <a:ext cx="5286375" cy="285750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4307,6 +4369,63 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1771650</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="class_zh_2">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10563225" y="857250"/>
+          <a:ext cx="5286375" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="00A6B8"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="A6A6A6"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="45720" tIns="0" rIns="45720" bIns="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1000" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:latin typeface="Arial"/>
+            </a:rPr>
+            <a:t>事件上下文</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
@@ -4320,8 +4439,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="shortcut_zh_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        <xdr:cNvPr id="4" name="shortcut_zh_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4377,8 +4496,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="shortcut_zh_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        <xdr:cNvPr id="5" name="shortcut_zh_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4434,8 +4553,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="shortcut_zh_geometry">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        <xdr:cNvPr id="6" name="shortcut_zh_geometry">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4491,8 +4610,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="shortcut_zh_overlay">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        <xdr:cNvPr id="7" name="shortcut_zh_overlay">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4548,8 +4667,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="shortcut_zh_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        <xdr:cNvPr id="8" name="shortcut_zh_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4605,8 +4724,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="shortcut_zh_fog">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        <xdr:cNvPr id="9" name="shortcut_zh_fog">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4662,8 +4781,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="shortcut_zh_math">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        <xdr:cNvPr id="10" name="shortcut_zh_math">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4719,8 +4838,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="shortcut_zh_event">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+        <xdr:cNvPr id="11" name="shortcut_zh_event">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4776,8 +4895,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="shortcut_zh_projectile">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+        <xdr:cNvPr id="12" name="shortcut_zh_projectile">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4833,8 +4952,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="shortcut_zh_turret">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+        <xdr:cNvPr id="13" name="shortcut_zh_turret">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4890,8 +5009,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="back_zh_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+        <xdr:cNvPr id="14" name="back_zh_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4931,8 +5050,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="back_zh_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+        <xdr:cNvPr id="15" name="back_zh_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -4972,8 +5091,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="back_zh_geometry">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+        <xdr:cNvPr id="16" name="back_zh_geometry">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5013,8 +5132,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="back_zh_overlay">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+        <xdr:cNvPr id="17" name="back_zh_overlay">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5054,8 +5173,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="back_zh_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+        <xdr:cNvPr id="18" name="back_zh_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5095,8 +5214,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="back_zh_fog">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+        <xdr:cNvPr id="19" name="back_zh_fog">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5136,8 +5255,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="19" name="back_zh_math">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
+        <xdr:cNvPr id="20" name="back_zh_math">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5177,8 +5296,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="20" name="back_zh_event">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
+        <xdr:cNvPr id="21" name="back_zh_event">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5218,8 +5337,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="back_zh_projectile">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
+        <xdr:cNvPr id="22" name="back_zh_projectile">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5259,8 +5378,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="back_zh_turret">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
+        <xdr:cNvPr id="23" name="back_zh_turret">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5300,8 +5419,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="shortcut_zh_custom_projectile_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
+        <xdr:cNvPr id="24" name="shortcut_zh_custom_projectile_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5357,8 +5476,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="shortcut_zh_custom_projectile_pattern">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
+        <xdr:cNvPr id="25" name="shortcut_zh_custom_projectile_pattern">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5414,8 +5533,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="shortcut_zh_custom_projectile_motion">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
+        <xdr:cNvPr id="26" name="shortcut_zh_custom_projectile_motion">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5471,8 +5590,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="shortcut_zh_custom_projectile_lifecycle">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
+        <xdr:cNvPr id="27" name="shortcut_zh_custom_projectile_lifecycle">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5528,8 +5647,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="shortcut_zh_custom_projectile_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
+        <xdr:cNvPr id="28" name="shortcut_zh_custom_projectile_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5585,8 +5704,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="shortcut_zh_custom_projectile_runtime">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
+        <xdr:cNvPr id="29" name="shortcut_zh_custom_projectile_runtime">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5642,8 +5761,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="shortcut_zh_custom_projectile_collision">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
+        <xdr:cNvPr id="30" name="shortcut_zh_custom_projectile_collision">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5699,8 +5818,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="shortcut_zh_custom_projectile_effect">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
+        <xdr:cNvPr id="31" name="shortcut_zh_custom_projectile_effect">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5756,8 +5875,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="shortcut_zh_custom_projectile_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
+        <xdr:cNvPr id="32" name="shortcut_zh_custom_projectile_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5813,8 +5932,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="32" name="back_zh_custom_projectile_core">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
+        <xdr:cNvPr id="33" name="back_zh_custom_projectile_core">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5854,8 +5973,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="33" name="back_zh_custom_projectile_pattern">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33"/>
+        <xdr:cNvPr id="34" name="back_zh_custom_projectile_pattern">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5895,8 +6014,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="34" name="back_zh_custom_projectile_motion">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
+        <xdr:cNvPr id="35" name="back_zh_custom_projectile_motion">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5936,8 +6055,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="35" name="back_zh_custom_projectile_lifecycle">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35"/>
+        <xdr:cNvPr id="36" name="back_zh_custom_projectile_lifecycle">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -5977,8 +6096,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="36" name="back_zh_custom_projectile_action">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
+        <xdr:cNvPr id="37" name="back_zh_custom_projectile_action">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6018,8 +6137,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="37" name="back_zh_custom_projectile_runtime">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
+        <xdr:cNvPr id="38" name="back_zh_custom_projectile_runtime">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6059,8 +6178,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="38" name="back_zh_custom_projectile_collision">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
+        <xdr:cNvPr id="39" name="back_zh_custom_projectile_collision">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6100,8 +6219,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="39" name="back_zh_custom_projectile_effect">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
+        <xdr:cNvPr id="40" name="back_zh_custom_projectile_effect">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId40"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6141,8 +6260,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="40" name="back_zh_custom_projectile_decal">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId40"/>
+        <xdr:cNvPr id="41" name="back_zh_custom_projectile_decal">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6182,8 +6301,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="41" name="shortcut_zh_event_tookdamage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41"/>
+        <xdr:cNvPr id="42" name="shortcut_zh_event_tookdamage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId42"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6239,8 +6358,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="42" name="shortcut_zh_event_queueitemadded">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId42"/>
+        <xdr:cNvPr id="43" name="shortcut_zh_event_queueitemadded">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6296,8 +6415,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="43" name="shortcut_zh_event_queueitemcancelled">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43"/>
+        <xdr:cNvPr id="44" name="shortcut_zh_event_queueitemcancelled">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId44"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6353,8 +6472,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="44" name="shortcut_zh_event_newwaypointgivenbyplayer">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId44"/>
+        <xdr:cNvPr id="45" name="shortcut_zh_event_newwaypointgivenbyplayer">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6410,8 +6529,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="45" name="shortcut_zh_event_teamchanged">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45"/>
+        <xdr:cNvPr id="46" name="shortcut_zh_event_teamchanged">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId46"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6467,8 +6586,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="46" name="shortcut_zh_event_teleported">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId46"/>
+        <xdr:cNvPr id="47" name="shortcut_zh_event_teleported">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6524,8 +6643,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="47" name="shortcut_zh_event_attachmentremoved">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47"/>
+        <xdr:cNvPr id="48" name="shortcut_zh_event_attachmentremoved">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId48"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6581,8 +6700,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="48" name="shortcut_zh_event_killedanyunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId48"/>
+        <xdr:cNvPr id="49" name="shortcut_zh_event_killedanyunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6638,8 +6757,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="49" name="shortcut_zh_event_queuedunitfinished">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49"/>
+        <xdr:cNvPr id="50" name="shortcut_zh_event_queuedunitfinished">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6695,8 +6814,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="50" name="shortcut_zh_event_touchtargetsuccess">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
+        <xdr:cNvPr id="51" name="shortcut_zh_event_touchtargetsuccess">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6752,8 +6871,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="51" name="shortcut_zh_event_transportingnewunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51"/>
+        <xdr:cNvPr id="52" name="shortcut_zh_event_transportingnewunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId52"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6809,8 +6928,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="52" name="shortcut_zh_event_transportunloadedorremovedunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId52"/>
+        <xdr:cNvPr id="53" name="shortcut_zh_event_transportunloadedorremovedunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6866,8 +6985,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="53" name="shortcut_zh_event_enteredtransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53"/>
+        <xdr:cNvPr id="54" name="shortcut_zh_event_enteredtransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId54"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6923,8 +7042,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="54" name="shortcut_zh_event_lefttransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId54"/>
+        <xdr:cNvPr id="55" name="shortcut_zh_event_lefttransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -6980,8 +7099,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="55" name="shortcut_zh_event_newmessage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
+        <xdr:cNvPr id="56" name="shortcut_zh_event_newmessage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId56"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7037,8 +7156,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="56" name="back_zh_event_tookdamage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId56"/>
+        <xdr:cNvPr id="57" name="back_zh_event_tookdamage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7078,8 +7197,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="57" name="back_zh_event_queueitemadded">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
+        <xdr:cNvPr id="58" name="back_zh_event_queueitemadded">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId58"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7119,8 +7238,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="58" name="back_zh_event_queueitemcancelled">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId58"/>
+        <xdr:cNvPr id="59" name="back_zh_event_queueitemcancelled">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7160,8 +7279,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="59" name="back_zh_event_newwaypointgivenbyplayer">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
+        <xdr:cNvPr id="60" name="back_zh_event_newwaypointgivenbyplayer">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId60"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7201,8 +7320,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="60" name="back_zh_event_teamchanged">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId60"/>
+        <xdr:cNvPr id="61" name="back_zh_event_teamchanged">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId61"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7242,8 +7361,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="61" name="back_zh_event_teleported">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId61"/>
+        <xdr:cNvPr id="62" name="back_zh_event_teleported">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId62"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7283,8 +7402,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="62" name="back_zh_event_attachmentremoved">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId62"/>
+        <xdr:cNvPr id="63" name="back_zh_event_attachmentremoved">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7324,8 +7443,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="63" name="back_zh_event_killedanyunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63"/>
+        <xdr:cNvPr id="64" name="back_zh_event_killedanyunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId64"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7365,8 +7484,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="64" name="back_zh_event_queuedunitfinished">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId64"/>
+        <xdr:cNvPr id="65" name="back_zh_event_queuedunitfinished">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId65"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7406,8 +7525,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="65" name="back_zh_event_touchtargetsuccess">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId65"/>
+        <xdr:cNvPr id="66" name="back_zh_event_touchtargetsuccess">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7447,8 +7566,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="66" name="back_zh_event_transportingnewunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
+        <xdr:cNvPr id="67" name="back_zh_event_transportingnewunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7488,8 +7607,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="67" name="back_zh_event_transportunloadedorremovedunit">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
+        <xdr:cNvPr id="68" name="back_zh_event_transportunloadedorremovedunit">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId68"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7529,8 +7648,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="68" name="back_zh_event_enteredtransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId68"/>
+        <xdr:cNvPr id="69" name="back_zh_event_enteredtransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7570,8 +7689,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="69" name="back_zh_event_lefttransport">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
+        <xdr:cNvPr id="70" name="back_zh_event_lefttransport">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -7611,8 +7730,8 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="70" name="back_zh_event_newmessage">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
+        <xdr:cNvPr id="71" name="back_zh_event_newmessage">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
         </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
@@ -8174,44 +8293,36 @@
       <c r="H2" s="7" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>CustomUnitMetadata</t>
-        </is>
-      </c>
+      <c r="A3" s="8" t="n"/>
       <c r="B3" s="8" t="n"/>
       <c r="C3" s="8" t="n"/>
       <c r="D3" s="8" t="n"/>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>CustomProjectile</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>CustomUnitMetadata sections</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
     </row>
     <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
+      <c r="B5" s="10" t="n"/>
       <c r="C5" s="11" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
@@ -16174,146 +16285,146 @@
       </c>
     </row>
     <row r="210" ht="24" customHeight="1">
-      <c r="A210" s="9" t="inlineStr">
+      <c r="A210" s="58" t="inlineStr">
         <is>
           <t>CustomProjectile sections</t>
         </is>
       </c>
-      <c r="B210" s="9" t="n"/>
-      <c r="C210" s="9" t="n"/>
-      <c r="D210" s="9" t="n"/>
-      <c r="E210" s="9" t="n"/>
-      <c r="F210" s="9" t="n"/>
-      <c r="G210" s="9" t="n"/>
-      <c r="H210" s="9" t="n"/>
+      <c r="B210" s="58" t="n"/>
+      <c r="C210" s="58" t="n"/>
+      <c r="D210" s="58" t="n"/>
+      <c r="E210" s="58" t="n"/>
+      <c r="F210" s="58" t="n"/>
+      <c r="G210" s="58" t="n"/>
+      <c r="H210" s="58" t="n"/>
     </row>
     <row r="211" ht="27" customHeight="1">
-      <c r="A211" s="9" t="inlineStr">
+      <c r="A211" s="58" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="B211" s="9" t="n"/>
-      <c r="C211" s="9" t="inlineStr">
+      <c r="B211" s="58" t="n"/>
+      <c r="C211" s="58" t="inlineStr">
         <is>
           <t>[pattern_NAME]</t>
         </is>
       </c>
-      <c r="D211" s="9" t="n"/>
-      <c r="E211" s="9" t="inlineStr">
+      <c r="D211" s="58" t="n"/>
+      <c r="E211" s="58" t="inlineStr">
         <is>
           <t>[motion]</t>
         </is>
       </c>
-      <c r="F211" s="9" t="n"/>
-      <c r="G211" s="9" t="inlineStr">
+      <c r="F211" s="58" t="n"/>
+      <c r="G211" s="58" t="inlineStr">
         <is>
           <t>[lifecycle]</t>
         </is>
       </c>
-      <c r="H211" s="9" t="n"/>
+      <c r="H211" s="58" t="n"/>
     </row>
     <row r="212" ht="27" customHeight="1">
-      <c r="A212" s="9" t="inlineStr">
+      <c r="A212" s="58" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="B212" s="9" t="n"/>
-      <c r="C212" s="9" t="inlineStr">
+      <c r="B212" s="58" t="n"/>
+      <c r="C212" s="58" t="inlineStr">
         <is>
           <t>CustomProjectile runtime expressions</t>
         </is>
       </c>
-      <c r="D212" s="9" t="n"/>
-      <c r="E212" s="9" t="inlineStr">
+      <c r="D212" s="58" t="n"/>
+      <c r="E212" s="58" t="inlineStr">
         <is>
           <t>[collision]</t>
         </is>
       </c>
-      <c r="F212" s="9" t="n"/>
-      <c r="G212" s="9" t="inlineStr">
+      <c r="F212" s="58" t="n"/>
+      <c r="G212" s="58" t="inlineStr">
         <is>
           <t>[effect_NAME]</t>
         </is>
       </c>
-      <c r="H212" s="9" t="n"/>
+      <c r="H212" s="58" t="n"/>
     </row>
     <row r="213" ht="27" customHeight="1">
-      <c r="A213" s="9" t="inlineStr">
+      <c r="A213" s="58" t="inlineStr">
         <is>
           <t>[decal_NAME]</t>
         </is>
       </c>
-      <c r="B213" s="9" t="n"/>
+      <c r="B213" s="58" t="n"/>
     </row>
     <row r="215" ht="34" customHeight="1">
-      <c r="A215" s="58" t="inlineStr">
+      <c r="A215" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B215" s="58" t="inlineStr">
+      <c r="B215" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C215" s="58" t="n"/>
-      <c r="D215" s="59" t="inlineStr">
+      <c r="C215" s="59" t="n"/>
+      <c r="D215" s="60" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="E215" s="58" t="inlineStr">
+      <c r="E215" s="59" t="inlineStr">
         <is>
           <t>Identity and schema fields for an independent CustomProjectile asset</t>
         </is>
       </c>
       <c r="F215" s="22" t="n"/>
       <c r="G215" s="23" t="n"/>
-      <c r="H215" s="59" t="inlineStr">
+      <c r="H215" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="216" ht="31" customHeight="1">
-      <c r="A216" s="60" t="inlineStr">
+      <c r="A216" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B216" s="60" t="inlineStr">
+      <c r="B216" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C216" s="60" t="inlineStr">
+      <c r="C216" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D216" s="60" t="inlineStr">
+      <c r="D216" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E216" s="60" t="inlineStr">
+      <c r="E216" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F216" s="60" t="inlineStr">
+      <c r="F216" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G216" s="60" t="inlineStr">
+      <c r="G216" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H216" s="60" t="inlineStr">
+      <c r="H216" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -16488,72 +16599,72 @@
       </c>
     </row>
     <row r="222" ht="34" customHeight="1">
-      <c r="A222" s="58" t="inlineStr">
+      <c r="A222" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B222" s="58" t="inlineStr">
+      <c r="B222" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C222" s="58" t="n"/>
-      <c r="D222" s="59" t="inlineStr">
+      <c r="C222" s="59" t="n"/>
+      <c r="D222" s="60" t="inlineStr">
         <is>
           <t>[pattern_NAME]</t>
         </is>
       </c>
-      <c r="E222" s="58" t="inlineStr">
+      <c r="E222" s="59" t="inlineStr">
         <is>
           <t>Deterministic same-tick layouts attached to this projectile asset</t>
         </is>
       </c>
       <c r="F222" s="22" t="n"/>
       <c r="G222" s="23" t="n"/>
-      <c r="H222" s="59" t="inlineStr">
+      <c r="H222" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="223" ht="31" customHeight="1">
-      <c r="A223" s="60" t="inlineStr">
+      <c r="A223" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B223" s="60" t="inlineStr">
+      <c r="B223" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C223" s="60" t="inlineStr">
+      <c r="C223" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D223" s="60" t="inlineStr">
+      <c r="D223" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E223" s="60" t="inlineStr">
+      <c r="E223" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F223" s="60" t="inlineStr">
+      <c r="F223" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G223" s="60" t="inlineStr">
+      <c r="G223" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H223" s="60" t="inlineStr">
+      <c r="H223" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -17064,72 +17175,72 @@
       </c>
     </row>
     <row r="237" ht="34" customHeight="1">
-      <c r="A237" s="58" t="inlineStr">
+      <c r="A237" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B237" s="58" t="inlineStr">
+      <c r="B237" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C237" s="58" t="n"/>
-      <c r="D237" s="59" t="inlineStr">
+      <c r="C237" s="59" t="n"/>
+      <c r="D237" s="60" t="inlineStr">
         <is>
           <t>[motion]</t>
         </is>
       </c>
-      <c r="E237" s="58" t="inlineStr">
+      <c r="E237" s="59" t="inlineStr">
         <is>
           <t>Live motion overrides evaluated during projectile flight</t>
         </is>
       </c>
       <c r="F237" s="22" t="n"/>
       <c r="G237" s="23" t="n"/>
-      <c r="H237" s="59" t="inlineStr">
+      <c r="H237" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="238" ht="31" customHeight="1">
-      <c r="A238" s="60" t="inlineStr">
+      <c r="A238" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B238" s="60" t="inlineStr">
+      <c r="B238" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C238" s="60" t="inlineStr">
+      <c r="C238" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D238" s="60" t="inlineStr">
+      <c r="D238" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E238" s="60" t="inlineStr">
+      <c r="E238" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F238" s="60" t="inlineStr">
+      <c r="F238" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G238" s="60" t="inlineStr">
+      <c r="G238" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H238" s="60" t="inlineStr">
+      <c r="H238" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -17388,72 +17499,72 @@
       </c>
     </row>
     <row r="246" ht="34" customHeight="1">
-      <c r="A246" s="58" t="inlineStr">
+      <c r="A246" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B246" s="58" t="inlineStr">
+      <c r="B246" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C246" s="58" t="n"/>
-      <c r="D246" s="59" t="inlineStr">
+      <c r="C246" s="59" t="n"/>
+      <c r="D246" s="60" t="inlineStr">
         <is>
           <t>[lifecycle]</t>
         </is>
       </c>
-      <c r="E246" s="58" t="inlineStr">
+      <c r="E246" s="59" t="inlineStr">
         <is>
           <t>Projectile-local actions invoked at lifecycle boundaries</t>
         </is>
       </c>
       <c r="F246" s="22" t="n"/>
       <c r="G246" s="23" t="n"/>
-      <c r="H246" s="59" t="inlineStr">
+      <c r="H246" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="247" ht="31" customHeight="1">
-      <c r="A247" s="60" t="inlineStr">
+      <c r="A247" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B247" s="60" t="inlineStr">
+      <c r="B247" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C247" s="60" t="inlineStr">
+      <c r="C247" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D247" s="60" t="inlineStr">
+      <c r="D247" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E247" s="60" t="inlineStr">
+      <c r="E247" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F247" s="60" t="inlineStr">
+      <c r="F247" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G247" s="60" t="inlineStr">
+      <c r="G247" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H247" s="60" t="inlineStr">
+      <c r="H247" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -17628,72 +17739,72 @@
       </c>
     </row>
     <row r="253" ht="34" customHeight="1">
-      <c r="A253" s="58" t="inlineStr">
+      <c r="A253" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B253" s="58" t="inlineStr">
+      <c r="B253" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C253" s="58" t="n"/>
-      <c r="D253" s="59" t="inlineStr">
+      <c r="C253" s="59" t="n"/>
+      <c r="D253" s="60" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="E253" s="58" t="inlineStr">
+      <c r="E253" s="59" t="inlineStr">
         <is>
           <t>Actions executed with the current projectile evaluation context</t>
         </is>
       </c>
       <c r="F253" s="22" t="n"/>
       <c r="G253" s="23" t="n"/>
-      <c r="H253" s="59" t="inlineStr">
+      <c r="H253" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="254" ht="31" customHeight="1">
-      <c r="A254" s="60" t="inlineStr">
+      <c r="A254" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B254" s="60" t="inlineStr">
+      <c r="B254" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C254" s="60" t="inlineStr">
+      <c r="C254" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D254" s="60" t="inlineStr">
+      <c r="D254" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E254" s="60" t="inlineStr">
+      <c r="E254" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F254" s="60" t="inlineStr">
+      <c r="F254" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G254" s="60" t="inlineStr">
+      <c r="G254" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H254" s="60" t="inlineStr">
+      <c r="H254" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -18078,72 +18189,72 @@
       </c>
     </row>
     <row r="265" ht="34" customHeight="1">
-      <c r="A265" s="58" t="inlineStr">
+      <c r="A265" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B265" s="58" t="inlineStr">
+      <c r="B265" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C265" s="58" t="n"/>
-      <c r="D265" s="59" t="inlineStr">
+      <c r="C265" s="59" t="n"/>
+      <c r="D265" s="60" t="inlineStr">
         <is>
           <t>CustomProjectile runtime expressions</t>
         </is>
       </c>
-      <c r="E265" s="58" t="inlineStr">
+      <c r="E265" s="59" t="inlineStr">
         <is>
           <t>Projectile values available inside dynamic expressions; not an INI section</t>
         </is>
       </c>
       <c r="F265" s="22" t="n"/>
       <c r="G265" s="23" t="n"/>
-      <c r="H265" s="59" t="inlineStr">
+      <c r="H265" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="266" ht="31" customHeight="1">
-      <c r="A266" s="60" t="inlineStr">
+      <c r="A266" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B266" s="60" t="inlineStr">
+      <c r="B266" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C266" s="60" t="inlineStr">
+      <c r="C266" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D266" s="60" t="inlineStr">
+      <c r="D266" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E266" s="60" t="inlineStr">
+      <c r="E266" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F266" s="60" t="inlineStr">
+      <c r="F266" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G266" s="60" t="inlineStr">
+      <c r="G266" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H266" s="60" t="inlineStr">
+      <c r="H266" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -18318,72 +18429,72 @@
       </c>
     </row>
     <row r="272" ht="34" customHeight="1">
-      <c r="A272" s="58" t="inlineStr">
+      <c r="A272" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B272" s="58" t="inlineStr">
+      <c r="B272" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C272" s="58" t="n"/>
-      <c r="D272" s="59" t="inlineStr">
+      <c r="C272" s="59" t="n"/>
+      <c r="D272" s="60" t="inlineStr">
         <is>
           <t>[collision]</t>
         </is>
       </c>
-      <c r="E272" s="58" t="inlineStr">
+      <c r="E272" s="59" t="inlineStr">
         <is>
           <t>Native unit contact and hover-path terrain collision</t>
         </is>
       </c>
       <c r="F272" s="22" t="n"/>
       <c r="G272" s="23" t="n"/>
-      <c r="H272" s="59" t="inlineStr">
+      <c r="H272" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="273" ht="31" customHeight="1">
-      <c r="A273" s="60" t="inlineStr">
+      <c r="A273" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B273" s="60" t="inlineStr">
+      <c r="B273" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C273" s="60" t="inlineStr">
+      <c r="C273" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D273" s="60" t="inlineStr">
+      <c r="D273" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E273" s="60" t="inlineStr">
+      <c r="E273" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F273" s="60" t="inlineStr">
+      <c r="F273" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G273" s="60" t="inlineStr">
+      <c r="G273" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H273" s="60" t="inlineStr">
+      <c r="H273" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -18894,72 +19005,72 @@
       </c>
     </row>
     <row r="287" ht="34" customHeight="1">
-      <c r="A287" s="58" t="inlineStr">
+      <c r="A287" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B287" s="58" t="inlineStr">
+      <c r="B287" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C287" s="58" t="n"/>
-      <c r="D287" s="59" t="inlineStr">
+      <c r="C287" s="59" t="n"/>
+      <c r="D287" s="60" t="inlineStr">
         <is>
           <t>[effect_NAME]</t>
         </is>
       </c>
-      <c r="E287" s="58" t="inlineStr">
+      <c r="E287" s="59" t="inlineStr">
         <is>
           <t>Native custom effects referenced by this projectile asset</t>
         </is>
       </c>
       <c r="F287" s="22" t="n"/>
       <c r="G287" s="23" t="n"/>
-      <c r="H287" s="59" t="inlineStr">
+      <c r="H287" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="288" ht="31" customHeight="1">
-      <c r="A288" s="60" t="inlineStr">
+      <c r="A288" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B288" s="60" t="inlineStr">
+      <c r="B288" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C288" s="60" t="inlineStr">
+      <c r="C288" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D288" s="60" t="inlineStr">
+      <c r="D288" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E288" s="60" t="inlineStr">
+      <c r="E288" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F288" s="60" t="inlineStr">
+      <c r="F288" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G288" s="60" t="inlineStr">
+      <c r="G288" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H288" s="60" t="inlineStr">
+      <c r="H288" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -19008,72 +19119,72 @@
       </c>
     </row>
     <row r="291" ht="34" customHeight="1">
-      <c r="A291" s="58" t="inlineStr">
+      <c r="A291" s="59" t="inlineStr">
         <is>
           <t>Catalog</t>
         </is>
       </c>
-      <c r="B291" s="58" t="inlineStr">
+      <c r="B291" s="59" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C291" s="58" t="n"/>
-      <c r="D291" s="59" t="inlineStr">
+      <c r="C291" s="59" t="n"/>
+      <c r="D291" s="60" t="inlineStr">
         <is>
           <t>[decal_NAME]</t>
         </is>
       </c>
-      <c r="E291" s="58" t="inlineStr">
+      <c r="E291" s="59" t="inlineStr">
         <is>
           <t>Native Decals anchored at the projectile's live world position</t>
         </is>
       </c>
       <c r="F291" s="22" t="n"/>
       <c r="G291" s="23" t="n"/>
-      <c r="H291" s="59" t="inlineStr">
+      <c r="H291" s="60" t="inlineStr">
         <is>
           <t>↑ Shortcuts</t>
         </is>
       </c>
     </row>
     <row r="292" ht="31" customHeight="1">
-      <c r="A292" s="60" t="inlineStr">
+      <c r="A292" s="61" t="inlineStr">
         <is>
           <t>Catalog Revision</t>
         </is>
       </c>
-      <c r="B292" s="60" t="inlineStr">
+      <c r="B292" s="61" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="C292" s="60" t="inlineStr">
+      <c r="C292" s="61" t="inlineStr">
         <is>
           <t>Value Type</t>
         </is>
       </c>
-      <c r="D292" s="60" t="inlineStr">
+      <c r="D292" s="61" t="inlineStr">
         <is>
           <t>Description and usage</t>
         </is>
       </c>
-      <c r="E292" s="60" t="inlineStr">
+      <c r="E292" s="61" t="inlineStr">
         <is>
           <t>Actual usage with examples</t>
         </is>
       </c>
-      <c r="F292" s="60" t="inlineStr">
+      <c r="F292" s="61" t="inlineStr">
         <is>
           <t>Extension Type</t>
         </is>
       </c>
-      <c r="G292" s="60" t="inlineStr">
+      <c r="G292" s="61" t="inlineStr">
         <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="H292" s="60" t="inlineStr">
+      <c r="H292" s="61" t="inlineStr">
         <is>
           <t>Multiplayer Impact</t>
         </is>
@@ -19122,32 +19233,32 @@
       </c>
     </row>
     <row r="295" ht="42" customHeight="1">
-      <c r="A295" s="61" t="inlineStr">
-        <is>
-          <t>Native autoTriggerOnEvent data extensions</t>
-        </is>
-      </c>
-      <c r="B295" s="61" t="n"/>
-      <c r="C295" s="61" t="n"/>
-      <c r="D295" s="61" t="n"/>
-      <c r="E295" s="61" t="n"/>
-      <c r="F295" s="61" t="n"/>
-      <c r="G295" s="61" t="n"/>
-      <c r="H295" s="61" t="n"/>
+      <c r="A295" s="62" t="inlineStr">
+        <is>
+          <t>EventContext — native autoTriggerOnEvent data extensions</t>
+        </is>
+      </c>
+      <c r="B295" s="62" t="n"/>
+      <c r="C295" s="62" t="n"/>
+      <c r="D295" s="62" t="n"/>
+      <c r="E295" s="62" t="n"/>
+      <c r="F295" s="62" t="n"/>
+      <c r="G295" s="62" t="n"/>
+      <c r="H295" s="62" t="n"/>
     </row>
     <row r="296" ht="28" customHeight="1">
-      <c r="A296" s="62" t="inlineStr">
+      <c r="A296" s="63" t="inlineStr">
         <is>
           <t>Event shortcuts — click to jump</t>
         </is>
       </c>
-      <c r="B296" s="62" t="n"/>
-      <c r="C296" s="62" t="n"/>
-      <c r="D296" s="62" t="n"/>
-      <c r="E296" s="62" t="n"/>
-      <c r="F296" s="62" t="n"/>
-      <c r="G296" s="62" t="n"/>
-      <c r="H296" s="62" t="n"/>
+      <c r="B296" s="63" t="n"/>
+      <c r="C296" s="63" t="n"/>
+      <c r="D296" s="63" t="n"/>
+      <c r="E296" s="63" t="n"/>
+      <c r="F296" s="63" t="n"/>
+      <c r="G296" s="63" t="n"/>
+      <c r="H296" s="63" t="n"/>
     </row>
     <row r="297" ht="27" customHeight="1">
       <c r="A297" s="17" t="inlineStr">
@@ -24822,7 +24933,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="76">
+  <mergeCells count="74">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E435:G435"/>
     <mergeCell ref="E297:F297"/>
@@ -24845,10 +24956,9 @@
     <mergeCell ref="E222:G222"/>
     <mergeCell ref="E369:G369"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="E3:H3"/>
     <mergeCell ref="E49:G49"/>
+    <mergeCell ref="E445:G445"/>
     <mergeCell ref="A212:B212"/>
-    <mergeCell ref="E445:G445"/>
     <mergeCell ref="E287:G287"/>
     <mergeCell ref="C212:D212"/>
     <mergeCell ref="E315:G315"/>
@@ -24887,7 +24997,6 @@
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E387:G387"/>
     <mergeCell ref="E212:F212"/>
-    <mergeCell ref="A3:D3"/>
     <mergeCell ref="E132:G132"/>
     <mergeCell ref="E141:G141"/>
     <mergeCell ref="G212:H212"/>
@@ -24955,44 +25064,36 @@
       <c r="H2" s="7" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>CustomUnitMetadata</t>
-        </is>
-      </c>
+      <c r="A3" s="8" t="n"/>
       <c r="B3" s="8" t="n"/>
       <c r="C3" s="8" t="n"/>
       <c r="D3" s="8" t="n"/>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>CustomProjectile</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>CustomUnitMetadata 节导航</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
     </row>
     <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
+      <c r="B5" s="10" t="n"/>
       <c r="C5" s="11" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
@@ -32955,146 +33056,146 @@
       </c>
     </row>
     <row r="210" ht="24" customHeight="1">
-      <c r="A210" s="9" t="inlineStr">
+      <c r="A210" s="58" t="inlineStr">
         <is>
           <t>CustomProjectile 节导航</t>
         </is>
       </c>
-      <c r="B210" s="9" t="n"/>
-      <c r="C210" s="9" t="n"/>
-      <c r="D210" s="9" t="n"/>
-      <c r="E210" s="9" t="n"/>
-      <c r="F210" s="9" t="n"/>
-      <c r="G210" s="9" t="n"/>
-      <c r="H210" s="9" t="n"/>
+      <c r="B210" s="58" t="n"/>
+      <c r="C210" s="58" t="n"/>
+      <c r="D210" s="58" t="n"/>
+      <c r="E210" s="58" t="n"/>
+      <c r="F210" s="58" t="n"/>
+      <c r="G210" s="58" t="n"/>
+      <c r="H210" s="58" t="n"/>
     </row>
     <row r="211" ht="27" customHeight="1">
-      <c r="A211" s="9" t="inlineStr">
+      <c r="A211" s="58" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="B211" s="9" t="n"/>
-      <c r="C211" s="9" t="inlineStr">
+      <c r="B211" s="58" t="n"/>
+      <c r="C211" s="58" t="inlineStr">
         <is>
           <t>[pattern_NAME]</t>
         </is>
       </c>
-      <c r="D211" s="9" t="n"/>
-      <c r="E211" s="9" t="inlineStr">
+      <c r="D211" s="58" t="n"/>
+      <c r="E211" s="58" t="inlineStr">
         <is>
           <t>[motion]</t>
         </is>
       </c>
-      <c r="F211" s="9" t="n"/>
-      <c r="G211" s="9" t="inlineStr">
+      <c r="F211" s="58" t="n"/>
+      <c r="G211" s="58" t="inlineStr">
         <is>
           <t>[lifecycle]</t>
         </is>
       </c>
-      <c r="H211" s="9" t="n"/>
+      <c r="H211" s="58" t="n"/>
     </row>
     <row r="212" ht="27" customHeight="1">
-      <c r="A212" s="9" t="inlineStr">
+      <c r="A212" s="58" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="B212" s="9" t="n"/>
-      <c r="C212" s="9" t="inlineStr">
+      <c r="B212" s="58" t="n"/>
+      <c r="C212" s="58" t="inlineStr">
         <is>
           <t>CustomProjectile 运行时表达式</t>
         </is>
       </c>
-      <c r="D212" s="9" t="n"/>
-      <c r="E212" s="9" t="inlineStr">
+      <c r="D212" s="58" t="n"/>
+      <c r="E212" s="58" t="inlineStr">
         <is>
           <t>[collision]</t>
         </is>
       </c>
-      <c r="F212" s="9" t="n"/>
-      <c r="G212" s="9" t="inlineStr">
+      <c r="F212" s="58" t="n"/>
+      <c r="G212" s="58" t="inlineStr">
         <is>
           <t>[effect_NAME]</t>
         </is>
       </c>
-      <c r="H212" s="9" t="n"/>
+      <c r="H212" s="58" t="n"/>
     </row>
     <row r="213" ht="27" customHeight="1">
-      <c r="A213" s="9" t="inlineStr">
+      <c r="A213" s="58" t="inlineStr">
         <is>
           <t>[decal_NAME]</t>
         </is>
       </c>
-      <c r="B213" s="9" t="n"/>
+      <c r="B213" s="58" t="n"/>
     </row>
     <row r="215" ht="34" customHeight="1">
-      <c r="A215" s="58" t="inlineStr">
+      <c r="A215" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B215" s="58" t="inlineStr">
+      <c r="B215" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C215" s="58" t="n"/>
-      <c r="D215" s="59" t="inlineStr">
+      <c r="C215" s="59" t="n"/>
+      <c r="D215" s="60" t="inlineStr">
         <is>
           <t>[core]</t>
         </is>
       </c>
-      <c r="E215" s="58" t="inlineStr">
+      <c r="E215" s="59" t="inlineStr">
         <is>
           <t>独立 CustomProjectile 资源的标识与格式字段</t>
         </is>
       </c>
       <c r="F215" s="22" t="n"/>
       <c r="G215" s="23" t="n"/>
-      <c r="H215" s="59" t="inlineStr">
+      <c r="H215" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="216" ht="31" customHeight="1">
-      <c r="A216" s="60" t="inlineStr">
+      <c r="A216" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B216" s="60" t="inlineStr">
+      <c r="B216" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C216" s="60" t="inlineStr">
+      <c r="C216" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D216" s="60" t="inlineStr">
+      <c r="D216" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E216" s="60" t="inlineStr">
+      <c r="E216" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F216" s="60" t="inlineStr">
+      <c r="F216" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G216" s="60" t="inlineStr">
+      <c r="G216" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H216" s="60" t="inlineStr">
+      <c r="H216" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -33269,72 +33370,72 @@
       </c>
     </row>
     <row r="222" ht="34" customHeight="1">
-      <c r="A222" s="58" t="inlineStr">
+      <c r="A222" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B222" s="58" t="inlineStr">
+      <c r="B222" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C222" s="58" t="n"/>
-      <c r="D222" s="59" t="inlineStr">
+      <c r="C222" s="59" t="n"/>
+      <c r="D222" s="60" t="inlineStr">
         <is>
           <t>[pattern_NAME]</t>
         </is>
       </c>
-      <c r="E222" s="58" t="inlineStr">
+      <c r="E222" s="59" t="inlineStr">
         <is>
           <t>附属于此弹体资源的确定性同帧弹幕排布</t>
         </is>
       </c>
       <c r="F222" s="22" t="n"/>
       <c r="G222" s="23" t="n"/>
-      <c r="H222" s="59" t="inlineStr">
+      <c r="H222" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="223" ht="31" customHeight="1">
-      <c r="A223" s="60" t="inlineStr">
+      <c r="A223" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B223" s="60" t="inlineStr">
+      <c r="B223" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C223" s="60" t="inlineStr">
+      <c r="C223" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D223" s="60" t="inlineStr">
+      <c r="D223" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E223" s="60" t="inlineStr">
+      <c r="E223" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F223" s="60" t="inlineStr">
+      <c r="F223" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G223" s="60" t="inlineStr">
+      <c r="G223" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H223" s="60" t="inlineStr">
+      <c r="H223" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -33845,72 +33946,72 @@
       </c>
     </row>
     <row r="237" ht="34" customHeight="1">
-      <c r="A237" s="58" t="inlineStr">
+      <c r="A237" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B237" s="58" t="inlineStr">
+      <c r="B237" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C237" s="58" t="n"/>
-      <c r="D237" s="59" t="inlineStr">
+      <c r="C237" s="59" t="n"/>
+      <c r="D237" s="60" t="inlineStr">
         <is>
           <t>[motion]</t>
         </is>
       </c>
-      <c r="E237" s="58" t="inlineStr">
+      <c r="E237" s="59" t="inlineStr">
         <is>
           <t>弹体飞行过程中持续求值的运动覆盖</t>
         </is>
       </c>
       <c r="F237" s="22" t="n"/>
       <c r="G237" s="23" t="n"/>
-      <c r="H237" s="59" t="inlineStr">
+      <c r="H237" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="238" ht="31" customHeight="1">
-      <c r="A238" s="60" t="inlineStr">
+      <c r="A238" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B238" s="60" t="inlineStr">
+      <c r="B238" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C238" s="60" t="inlineStr">
+      <c r="C238" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D238" s="60" t="inlineStr">
+      <c r="D238" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E238" s="60" t="inlineStr">
+      <c r="E238" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F238" s="60" t="inlineStr">
+      <c r="F238" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G238" s="60" t="inlineStr">
+      <c r="G238" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H238" s="60" t="inlineStr">
+      <c r="H238" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -34169,72 +34270,72 @@
       </c>
     </row>
     <row r="246" ht="34" customHeight="1">
-      <c r="A246" s="58" t="inlineStr">
+      <c r="A246" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B246" s="58" t="inlineStr">
+      <c r="B246" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C246" s="58" t="n"/>
-      <c r="D246" s="59" t="inlineStr">
+      <c r="C246" s="59" t="n"/>
+      <c r="D246" s="60" t="inlineStr">
         <is>
           <t>[lifecycle]</t>
         </is>
       </c>
-      <c r="E246" s="58" t="inlineStr">
+      <c r="E246" s="59" t="inlineStr">
         <is>
           <t>在弹体生命周期节点触发的局部动作</t>
         </is>
       </c>
       <c r="F246" s="22" t="n"/>
       <c r="G246" s="23" t="n"/>
-      <c r="H246" s="59" t="inlineStr">
+      <c r="H246" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="247" ht="31" customHeight="1">
-      <c r="A247" s="60" t="inlineStr">
+      <c r="A247" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B247" s="60" t="inlineStr">
+      <c r="B247" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C247" s="60" t="inlineStr">
+      <c r="C247" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D247" s="60" t="inlineStr">
+      <c r="D247" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E247" s="60" t="inlineStr">
+      <c r="E247" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F247" s="60" t="inlineStr">
+      <c r="F247" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G247" s="60" t="inlineStr">
+      <c r="G247" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H247" s="60" t="inlineStr">
+      <c r="H247" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -34409,72 +34510,72 @@
       </c>
     </row>
     <row r="253" ht="34" customHeight="1">
-      <c r="A253" s="58" t="inlineStr">
+      <c r="A253" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B253" s="58" t="inlineStr">
+      <c r="B253" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C253" s="58" t="n"/>
-      <c r="D253" s="59" t="inlineStr">
+      <c r="C253" s="59" t="n"/>
+      <c r="D253" s="60" t="inlineStr">
         <is>
           <t>[action_NAME] / [hiddenAction_NAME]</t>
         </is>
       </c>
-      <c r="E253" s="58" t="inlineStr">
+      <c r="E253" s="59" t="inlineStr">
         <is>
           <t>在当前弹体求值上下文中执行的动作</t>
         </is>
       </c>
       <c r="F253" s="22" t="n"/>
       <c r="G253" s="23" t="n"/>
-      <c r="H253" s="59" t="inlineStr">
+      <c r="H253" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="254" ht="31" customHeight="1">
-      <c r="A254" s="60" t="inlineStr">
+      <c r="A254" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B254" s="60" t="inlineStr">
+      <c r="B254" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C254" s="60" t="inlineStr">
+      <c r="C254" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D254" s="60" t="inlineStr">
+      <c r="D254" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E254" s="60" t="inlineStr">
+      <c r="E254" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F254" s="60" t="inlineStr">
+      <c r="F254" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G254" s="60" t="inlineStr">
+      <c r="G254" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H254" s="60" t="inlineStr">
+      <c r="H254" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -34859,72 +34960,72 @@
       </c>
     </row>
     <row r="265" ht="34" customHeight="1">
-      <c r="A265" s="58" t="inlineStr">
+      <c r="A265" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B265" s="58" t="inlineStr">
+      <c r="B265" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C265" s="58" t="n"/>
-      <c r="D265" s="59" t="inlineStr">
+      <c r="C265" s="59" t="n"/>
+      <c r="D265" s="60" t="inlineStr">
         <is>
           <t>CustomProjectile 运行时表达式</t>
         </is>
       </c>
-      <c r="E265" s="58" t="inlineStr">
+      <c r="E265" s="59" t="inlineStr">
         <is>
           <t>动态表达式中可读取的弹体值；这不是一个 INI 节</t>
         </is>
       </c>
       <c r="F265" s="22" t="n"/>
       <c r="G265" s="23" t="n"/>
-      <c r="H265" s="59" t="inlineStr">
+      <c r="H265" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="266" ht="31" customHeight="1">
-      <c r="A266" s="60" t="inlineStr">
+      <c r="A266" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B266" s="60" t="inlineStr">
+      <c r="B266" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C266" s="60" t="inlineStr">
+      <c r="C266" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D266" s="60" t="inlineStr">
+      <c r="D266" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E266" s="60" t="inlineStr">
+      <c r="E266" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F266" s="60" t="inlineStr">
+      <c r="F266" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G266" s="60" t="inlineStr">
+      <c r="G266" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H266" s="60" t="inlineStr">
+      <c r="H266" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -35099,72 +35200,72 @@
       </c>
     </row>
     <row r="272" ht="34" customHeight="1">
-      <c r="A272" s="58" t="inlineStr">
+      <c r="A272" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B272" s="58" t="inlineStr">
+      <c r="B272" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C272" s="58" t="n"/>
-      <c r="D272" s="59" t="inlineStr">
+      <c r="C272" s="59" t="n"/>
+      <c r="D272" s="60" t="inlineStr">
         <is>
           <t>[collision]</t>
         </is>
       </c>
-      <c r="E272" s="58" t="inlineStr">
+      <c r="E272" s="59" t="inlineStr">
         <is>
           <t>原版单位接触与 hover 寻路地形碰撞</t>
         </is>
       </c>
       <c r="F272" s="22" t="n"/>
       <c r="G272" s="23" t="n"/>
-      <c r="H272" s="59" t="inlineStr">
+      <c r="H272" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="273" ht="31" customHeight="1">
-      <c r="A273" s="60" t="inlineStr">
+      <c r="A273" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B273" s="60" t="inlineStr">
+      <c r="B273" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C273" s="60" t="inlineStr">
+      <c r="C273" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D273" s="60" t="inlineStr">
+      <c r="D273" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E273" s="60" t="inlineStr">
+      <c r="E273" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F273" s="60" t="inlineStr">
+      <c r="F273" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G273" s="60" t="inlineStr">
+      <c r="G273" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H273" s="60" t="inlineStr">
+      <c r="H273" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -35675,72 +35776,72 @@
       </c>
     </row>
     <row r="287" ht="34" customHeight="1">
-      <c r="A287" s="58" t="inlineStr">
+      <c r="A287" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B287" s="58" t="inlineStr">
+      <c r="B287" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C287" s="58" t="n"/>
-      <c r="D287" s="59" t="inlineStr">
+      <c r="C287" s="59" t="n"/>
+      <c r="D287" s="60" t="inlineStr">
         <is>
           <t>[effect_NAME]</t>
         </is>
       </c>
-      <c r="E287" s="58" t="inlineStr">
+      <c r="E287" s="59" t="inlineStr">
         <is>
           <t>供此弹体资源引用的原版自定义特效</t>
         </is>
       </c>
       <c r="F287" s="22" t="n"/>
       <c r="G287" s="23" t="n"/>
-      <c r="H287" s="59" t="inlineStr">
+      <c r="H287" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="288" ht="31" customHeight="1">
-      <c r="A288" s="60" t="inlineStr">
+      <c r="A288" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B288" s="60" t="inlineStr">
+      <c r="B288" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C288" s="60" t="inlineStr">
+      <c r="C288" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D288" s="60" t="inlineStr">
+      <c r="D288" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E288" s="60" t="inlineStr">
+      <c r="E288" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F288" s="60" t="inlineStr">
+      <c r="F288" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G288" s="60" t="inlineStr">
+      <c r="G288" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H288" s="60" t="inlineStr">
+      <c r="H288" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -35789,72 +35890,72 @@
       </c>
     </row>
     <row r="291" ht="34" customHeight="1">
-      <c r="A291" s="58" t="inlineStr">
+      <c r="A291" s="59" t="inlineStr">
         <is>
           <t>目录</t>
         </is>
       </c>
-      <c r="B291" s="58" t="inlineStr">
+      <c r="B291" s="59" t="inlineStr">
         <is>
           <t>节</t>
         </is>
       </c>
-      <c r="C291" s="58" t="n"/>
-      <c r="D291" s="59" t="inlineStr">
+      <c r="C291" s="59" t="n"/>
+      <c r="D291" s="60" t="inlineStr">
         <is>
           <t>[decal_NAME]</t>
         </is>
       </c>
-      <c r="E291" s="58" t="inlineStr">
+      <c r="E291" s="59" t="inlineStr">
         <is>
           <t>锚定在弹体实时世界坐标的原版 Decal</t>
         </is>
       </c>
       <c r="F291" s="22" t="n"/>
       <c r="G291" s="23" t="n"/>
-      <c r="H291" s="59" t="inlineStr">
+      <c r="H291" s="60" t="inlineStr">
         <is>
           <t>↑ 返回节导航</t>
         </is>
       </c>
     </row>
     <row r="292" ht="31" customHeight="1">
-      <c r="A292" s="60" t="inlineStr">
+      <c r="A292" s="61" t="inlineStr">
         <is>
           <t>目录修订</t>
         </is>
       </c>
-      <c r="B292" s="60" t="inlineStr">
+      <c r="B292" s="61" t="inlineStr">
         <is>
           <t>代码</t>
         </is>
       </c>
-      <c r="C292" s="60" t="inlineStr">
+      <c r="C292" s="61" t="inlineStr">
         <is>
           <t>值类型</t>
         </is>
       </c>
-      <c r="D292" s="60" t="inlineStr">
+      <c r="D292" s="61" t="inlineStr">
         <is>
           <t>说明与用法</t>
         </is>
       </c>
-      <c r="E292" s="60" t="inlineStr">
+      <c r="E292" s="61" t="inlineStr">
         <is>
           <t>实际用法与示例</t>
         </is>
       </c>
-      <c r="F292" s="60" t="inlineStr">
+      <c r="F292" s="61" t="inlineStr">
         <is>
           <t>扩展类型</t>
         </is>
       </c>
-      <c r="G292" s="60" t="inlineStr">
+      <c r="G292" s="61" t="inlineStr">
         <is>
           <t>默认值</t>
         </is>
       </c>
-      <c r="H292" s="60" t="inlineStr">
+      <c r="H292" s="61" t="inlineStr">
         <is>
           <t>联机影响</t>
         </is>
@@ -35903,32 +36004,32 @@
       </c>
     </row>
     <row r="295" ht="42" customHeight="1">
-      <c r="A295" s="61" t="inlineStr">
-        <is>
-          <t>原版 autoTriggerOnEvent 事件数据扩展</t>
-        </is>
-      </c>
-      <c r="B295" s="61" t="n"/>
-      <c r="C295" s="61" t="n"/>
-      <c r="D295" s="61" t="n"/>
-      <c r="E295" s="61" t="n"/>
-      <c r="F295" s="61" t="n"/>
-      <c r="G295" s="61" t="n"/>
-      <c r="H295" s="61" t="n"/>
+      <c r="A295" s="62" t="inlineStr">
+        <is>
+          <t>事件上下文——原版 autoTriggerOnEvent 事件数据扩展</t>
+        </is>
+      </c>
+      <c r="B295" s="62" t="n"/>
+      <c r="C295" s="62" t="n"/>
+      <c r="D295" s="62" t="n"/>
+      <c r="E295" s="62" t="n"/>
+      <c r="F295" s="62" t="n"/>
+      <c r="G295" s="62" t="n"/>
+      <c r="H295" s="62" t="n"/>
     </row>
     <row r="296" ht="28" customHeight="1">
-      <c r="A296" s="62" t="inlineStr">
+      <c r="A296" s="63" t="inlineStr">
         <is>
           <t>事件快捷导航——点击即可跳转</t>
         </is>
       </c>
-      <c r="B296" s="62" t="n"/>
-      <c r="C296" s="62" t="n"/>
-      <c r="D296" s="62" t="n"/>
-      <c r="E296" s="62" t="n"/>
-      <c r="F296" s="62" t="n"/>
-      <c r="G296" s="62" t="n"/>
-      <c r="H296" s="62" t="n"/>
+      <c r="B296" s="63" t="n"/>
+      <c r="C296" s="63" t="n"/>
+      <c r="D296" s="63" t="n"/>
+      <c r="E296" s="63" t="n"/>
+      <c r="F296" s="63" t="n"/>
+      <c r="G296" s="63" t="n"/>
+      <c r="H296" s="63" t="n"/>
     </row>
     <row r="297" ht="27" customHeight="1">
       <c r="A297" s="17" t="inlineStr">
@@ -41603,7 +41704,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="76">
+  <mergeCells count="74">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E435:G435"/>
     <mergeCell ref="E297:F297"/>
@@ -41626,10 +41727,9 @@
     <mergeCell ref="E222:G222"/>
     <mergeCell ref="E369:G369"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="E3:H3"/>
     <mergeCell ref="E49:G49"/>
+    <mergeCell ref="E445:G445"/>
     <mergeCell ref="A212:B212"/>
-    <mergeCell ref="E445:G445"/>
     <mergeCell ref="E287:G287"/>
     <mergeCell ref="C212:D212"/>
     <mergeCell ref="E315:G315"/>
@@ -41668,7 +41768,6 @@
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E387:G387"/>
     <mergeCell ref="E212:F212"/>
-    <mergeCell ref="A3:D3"/>
     <mergeCell ref="E132:G132"/>
     <mergeCell ref="E141:G141"/>
     <mergeCell ref="G212:H212"/>

</xml_diff>

<commit_message>
Prepare Rusted Fabric 0.4.3 release
</commit_message>
<xml_diff>
--- a/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
+++ b/official-mods/ini-essentials/docs/INI Essentials Unit Modding Reference.xlsx
@@ -8064,7 +8064,7 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INI Essentials v0.3.0 Unit Modding Reference</t>
+          <t>INI Essentials v0.3.1 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -8078,7 +8078,7 @@
     <row r="3" ht="27" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Current mod version / 当前模组版本: 0.3.0</t>
+          <t>Current mod version / 当前模组版本: 0.3.1</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -8267,7 +8267,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials v0.3.0 Unit Modding Reference</t>
+          <t>INI Essentials v0.3.1 Unit Modding Reference</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>
@@ -25122,7 +25122,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>INI Essentials v0.3.0 单位模组代码表</t>
+          <t>INI Essentials v0.3.1 单位模组代码表</t>
         </is>
       </c>
       <c r="B1" s="6" t="n"/>

</xml_diff>